<commit_message>
Update dashboard UI and payment received
</commit_message>
<xml_diff>
--- a/Fees Details 2024-25.xlsx
+++ b/Fees Details 2024-25.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="197">
   <si>
     <t>ROOMS</t>
   </si>
@@ -42,6 +42,9 @@
   </si>
   <si>
     <t>outstanding fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Payment Received</t>
   </si>
   <si>
     <t>NAKUL PARAKH</t>
@@ -2256,7 +2259,7 @@
     <col min="7" max="7" width="32.2962962962963" style="3" customWidth="1"/>
     <col min="8" max="8" width="9.68518518518519" style="2" customWidth="1"/>
     <col min="9" max="9" width="22.0833333333333" style="4" customWidth="1"/>
-    <col min="10" max="10" width="11.3333333333333" style="4" customWidth="1"/>
+    <col min="10" max="10" width="19.5" style="4" customWidth="1"/>
     <col min="11" max="11" width="12.3333333333333" style="4" customWidth="1"/>
     <col min="12" max="12" width="16.3333333333333" style="4" customWidth="1"/>
     <col min="13" max="13" width="10.3333333333333" style="4" customWidth="1"/>
@@ -2289,7 +2292,9 @@
       <c r="I2" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="10"/>
+      <c r="J2" s="10" t="s">
+        <v>5</v>
+      </c>
       <c r="K2" s="10"/>
       <c r="L2" s="10"/>
       <c r="M2" s="10"/>
@@ -2311,18 +2316,20 @@
         <v>1</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" s="19">
         <v>1234567891</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I3" s="20">
         <v>10000</v>
       </c>
-      <c r="J3" s="21"/>
+      <c r="J3" s="21">
+        <v>85000</v>
+      </c>
       <c r="K3" s="21"/>
       <c r="L3" s="21"/>
       <c r="M3" s="22"/>
@@ -2342,18 +2349,20 @@
         <v>2</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4" s="19">
         <v>1234567892</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I4" s="20">
         <v>10001</v>
       </c>
-      <c r="J4" s="21"/>
+      <c r="J4" s="21">
+        <v>85001</v>
+      </c>
       <c r="K4" s="21"/>
       <c r="L4" s="21"/>
       <c r="M4" s="21"/>
@@ -2373,18 +2382,20 @@
         <v>3</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G5" s="19">
         <v>1234567893</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I5" s="20">
         <v>10002</v>
       </c>
-      <c r="J5" s="21"/>
+      <c r="J5" s="21">
+        <v>85002</v>
+      </c>
       <c r="K5" s="21"/>
       <c r="L5" s="21"/>
       <c r="M5" s="21"/>
@@ -2404,18 +2415,20 @@
         <v>4</v>
       </c>
       <c r="F6" s="28" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6" s="19">
         <v>1234567894</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I6" s="20">
         <v>10003</v>
       </c>
-      <c r="J6" s="21"/>
+      <c r="J6" s="21">
+        <v>85003</v>
+      </c>
       <c r="K6" s="21"/>
       <c r="L6" s="21"/>
       <c r="M6" s="21"/>
@@ -2437,18 +2450,20 @@
         <v>1</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G7" s="19">
         <v>1234567895</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I7" s="20">
         <v>10004</v>
       </c>
-      <c r="J7" s="32"/>
+      <c r="J7" s="21">
+        <v>85004</v>
+      </c>
       <c r="K7" s="32"/>
       <c r="L7" s="32"/>
       <c r="M7" s="32"/>
@@ -2468,18 +2483,20 @@
         <v>2</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G8" s="19">
         <v>1234567896</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I8" s="20">
         <v>10005</v>
       </c>
-      <c r="J8" s="21"/>
+      <c r="J8" s="21">
+        <v>85005</v>
+      </c>
       <c r="K8" s="21"/>
       <c r="L8" s="21"/>
       <c r="M8" s="21"/>
@@ -2499,18 +2516,20 @@
         <v>3</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G9" s="19">
         <v>1234567897</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I9" s="20">
         <v>10006</v>
       </c>
-      <c r="J9" s="21"/>
+      <c r="J9" s="21">
+        <v>85006</v>
+      </c>
       <c r="K9" s="21"/>
       <c r="L9" s="21"/>
       <c r="M9" s="21"/>
@@ -2530,18 +2549,20 @@
         <v>4</v>
       </c>
       <c r="F10" s="34" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G10" s="19">
         <v>1234567898</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I10" s="20">
         <v>10007</v>
       </c>
-      <c r="J10" s="35"/>
+      <c r="J10" s="21">
+        <v>85007</v>
+      </c>
       <c r="K10" s="35"/>
       <c r="L10" s="35"/>
       <c r="M10" s="35"/>
@@ -2563,18 +2584,20 @@
         <v>1</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G11" s="19">
         <v>1234567899</v>
       </c>
       <c r="H11" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I11" s="20">
         <v>10008</v>
       </c>
-      <c r="J11" s="32"/>
+      <c r="J11" s="21">
+        <v>85008</v>
+      </c>
       <c r="K11" s="32"/>
       <c r="L11" s="32"/>
       <c r="M11" s="32"/>
@@ -2594,18 +2617,20 @@
         <v>2</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G12" s="19">
         <v>1234567900</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I12" s="20">
         <v>10009</v>
       </c>
-      <c r="J12" s="21"/>
+      <c r="J12" s="21">
+        <v>85009</v>
+      </c>
       <c r="K12" s="21"/>
       <c r="L12" s="21"/>
       <c r="M12" s="21"/>
@@ -2625,18 +2650,20 @@
         <v>3</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G13" s="19">
         <v>1234567901</v>
       </c>
       <c r="H13" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I13" s="20">
         <v>10010</v>
       </c>
-      <c r="J13" s="21"/>
+      <c r="J13" s="21">
+        <v>85010</v>
+      </c>
       <c r="K13" s="21"/>
       <c r="L13" s="21"/>
       <c r="M13" s="21"/>
@@ -2656,18 +2683,20 @@
         <v>4</v>
       </c>
       <c r="F14" s="38" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G14" s="19">
         <v>1234567902</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I14" s="20">
         <v>10011</v>
       </c>
-      <c r="J14" s="39"/>
+      <c r="J14" s="21">
+        <v>85011</v>
+      </c>
       <c r="K14" s="39"/>
       <c r="L14" s="39"/>
       <c r="M14" s="39"/>
@@ -2685,18 +2714,20 @@
       <c r="D15" s="24"/>
       <c r="E15" s="30"/>
       <c r="F15" s="40" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G15" s="19">
         <v>1234567903</v>
       </c>
       <c r="H15" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I15" s="20">
         <v>10012</v>
       </c>
-      <c r="J15" s="21"/>
+      <c r="J15" s="21">
+        <v>85012</v>
+      </c>
       <c r="K15" s="21"/>
       <c r="L15" s="21"/>
       <c r="M15" s="21"/>
@@ -2718,18 +2749,20 @@
         <v>1</v>
       </c>
       <c r="F16" s="41" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G16" s="19">
         <v>1234567904</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I16" s="20">
         <v>10013</v>
       </c>
-      <c r="J16" s="32"/>
+      <c r="J16" s="21">
+        <v>85013</v>
+      </c>
       <c r="K16" s="32"/>
       <c r="L16" s="32"/>
       <c r="M16" s="42"/>
@@ -2749,18 +2782,20 @@
         <v>2</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G17" s="19">
         <v>1234567905</v>
       </c>
       <c r="H17" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I17" s="20">
         <v>10014</v>
       </c>
-      <c r="J17" s="21"/>
+      <c r="J17" s="21">
+        <v>85014</v>
+      </c>
       <c r="K17" s="21"/>
       <c r="L17" s="21"/>
       <c r="M17" s="21"/>
@@ -2780,18 +2815,20 @@
         <v>3</v>
       </c>
       <c r="F18" s="38" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G18" s="19">
         <v>1234567906</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I18" s="20">
         <v>10015</v>
       </c>
-      <c r="J18" s="21"/>
+      <c r="J18" s="21">
+        <v>85015</v>
+      </c>
       <c r="K18" s="21"/>
       <c r="L18" s="21"/>
       <c r="M18" s="21"/>
@@ -2811,18 +2848,20 @@
         <v>4</v>
       </c>
       <c r="F19" s="43" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G19" s="19">
         <v>1234567907</v>
       </c>
       <c r="H19" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I19" s="20">
         <v>10016</v>
       </c>
-      <c r="J19" s="35"/>
+      <c r="J19" s="21">
+        <v>85016</v>
+      </c>
       <c r="K19" s="35"/>
       <c r="L19" s="35"/>
       <c r="M19" s="35"/>
@@ -2844,18 +2883,20 @@
         <v>1</v>
       </c>
       <c r="F20" s="44" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G20" s="19">
         <v>1234567908</v>
       </c>
       <c r="H20" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I20" s="20">
         <v>10017</v>
       </c>
-      <c r="J20" s="32"/>
+      <c r="J20" s="21">
+        <v>85017</v>
+      </c>
       <c r="K20" s="32"/>
       <c r="L20" s="32"/>
       <c r="M20" s="32"/>
@@ -2875,18 +2916,20 @@
         <v>2</v>
       </c>
       <c r="F21" s="44" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G21" s="19">
         <v>1234567909</v>
       </c>
       <c r="H21" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I21" s="20">
         <v>10018</v>
       </c>
-      <c r="J21" s="21"/>
+      <c r="J21" s="21">
+        <v>85018</v>
+      </c>
       <c r="K21" s="21"/>
       <c r="L21" s="21"/>
       <c r="M21" s="21"/>
@@ -2906,18 +2949,20 @@
         <v>3</v>
       </c>
       <c r="F22" s="46" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G22" s="19">
         <v>1234567910</v>
       </c>
       <c r="H22" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I22" s="20">
         <v>10019</v>
       </c>
-      <c r="J22" s="21"/>
+      <c r="J22" s="21">
+        <v>85019</v>
+      </c>
       <c r="K22" s="21"/>
       <c r="L22" s="21"/>
       <c r="M22" s="21"/>
@@ -2937,18 +2982,20 @@
         <v>4</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G23" s="19">
         <v>1234567911</v>
       </c>
       <c r="H23" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I23" s="20">
         <v>10020</v>
       </c>
-      <c r="J23" s="39"/>
+      <c r="J23" s="21">
+        <v>85020</v>
+      </c>
       <c r="K23" s="39"/>
       <c r="L23" s="39"/>
       <c r="M23" s="39"/>
@@ -2966,18 +3013,20 @@
       <c r="D24" s="24"/>
       <c r="E24" s="47"/>
       <c r="F24" s="40" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G24" s="19">
         <v>1234567912</v>
       </c>
       <c r="H24" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I24" s="20">
         <v>10021</v>
       </c>
-      <c r="J24" s="21"/>
+      <c r="J24" s="21">
+        <v>85021</v>
+      </c>
       <c r="K24" s="21"/>
       <c r="L24" s="21"/>
       <c r="M24" s="21"/>
@@ -2999,18 +3048,20 @@
         <v>1</v>
       </c>
       <c r="F25" s="48" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G25" s="19">
         <v>1234567913</v>
       </c>
       <c r="H25" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I25" s="20">
         <v>10022</v>
       </c>
-      <c r="J25" s="32"/>
+      <c r="J25" s="21">
+        <v>85022</v>
+      </c>
       <c r="K25" s="32"/>
       <c r="L25" s="32"/>
       <c r="M25" s="32"/>
@@ -3030,18 +3081,20 @@
         <v>2</v>
       </c>
       <c r="F26" s="49" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G26" s="19">
         <v>1234567914</v>
       </c>
       <c r="H26" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I26" s="20">
         <v>10023</v>
       </c>
-      <c r="J26" s="21"/>
+      <c r="J26" s="21">
+        <v>85023</v>
+      </c>
       <c r="K26" s="21"/>
       <c r="L26" s="21"/>
       <c r="M26" s="21"/>
@@ -3061,18 +3114,20 @@
         <v>3</v>
       </c>
       <c r="F27" s="50" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G27" s="19">
         <v>1234567915</v>
       </c>
       <c r="H27" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I27" s="20">
         <v>10024</v>
       </c>
-      <c r="J27" s="21"/>
+      <c r="J27" s="21">
+        <v>85024</v>
+      </c>
       <c r="K27" s="21"/>
       <c r="L27" s="21"/>
       <c r="M27" s="21"/>
@@ -3092,18 +3147,20 @@
         <v>4</v>
       </c>
       <c r="F28" s="34" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G28" s="19">
         <v>1234567916</v>
       </c>
       <c r="H28" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I28" s="20">
         <v>10025</v>
       </c>
-      <c r="J28" s="35"/>
+      <c r="J28" s="21">
+        <v>85025</v>
+      </c>
       <c r="K28" s="35"/>
       <c r="L28" s="35"/>
       <c r="M28" s="35"/>
@@ -3125,18 +3182,20 @@
         <v>1</v>
       </c>
       <c r="F29" s="37" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G29" s="19">
         <v>1234567917</v>
       </c>
       <c r="H29" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I29" s="20">
         <v>10026</v>
       </c>
-      <c r="J29" s="32"/>
+      <c r="J29" s="21">
+        <v>85026</v>
+      </c>
       <c r="K29" s="32"/>
       <c r="L29" s="32"/>
       <c r="M29" s="32"/>
@@ -3156,18 +3215,20 @@
         <v>2</v>
       </c>
       <c r="F30" s="51" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G30" s="19">
         <v>1234567918</v>
       </c>
       <c r="H30" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I30" s="20">
         <v>10027</v>
       </c>
-      <c r="J30" s="21"/>
+      <c r="J30" s="21">
+        <v>85027</v>
+      </c>
       <c r="K30" s="21"/>
       <c r="L30" s="21"/>
       <c r="M30" s="21"/>
@@ -3187,18 +3248,20 @@
         <v>3</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G31" s="19">
         <v>1234567919</v>
       </c>
       <c r="H31" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I31" s="20">
         <v>10028</v>
       </c>
-      <c r="J31" s="21"/>
+      <c r="J31" s="21">
+        <v>85028</v>
+      </c>
       <c r="K31" s="21"/>
       <c r="L31" s="21"/>
       <c r="M31" s="21"/>
@@ -3218,18 +3281,20 @@
         <v>4</v>
       </c>
       <c r="F32" s="52" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G32" s="19">
         <v>1234567920</v>
       </c>
       <c r="H32" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I32" s="20">
         <v>10029</v>
       </c>
-      <c r="J32" s="21"/>
+      <c r="J32" s="21">
+        <v>85029</v>
+      </c>
       <c r="K32" s="21"/>
       <c r="L32" s="21"/>
       <c r="M32" s="21"/>
@@ -3249,18 +3314,20 @@
         <v>5</v>
       </c>
       <c r="F33" s="53" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G33" s="19">
         <v>1234567921</v>
       </c>
       <c r="H33" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I33" s="20">
         <v>10030</v>
       </c>
-      <c r="J33" s="39"/>
+      <c r="J33" s="21">
+        <v>85030</v>
+      </c>
       <c r="K33" s="21"/>
       <c r="L33" s="39"/>
       <c r="M33" s="39"/>
@@ -3278,16 +3345,19 @@
       <c r="D34" s="24"/>
       <c r="E34" s="30"/>
       <c r="F34" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G34" s="19">
         <v>1234567922</v>
       </c>
       <c r="H34" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I34" s="20">
         <v>10031</v>
+      </c>
+      <c r="J34" s="21">
+        <v>85031</v>
       </c>
     </row>
     <row r="35" ht="17.1" spans="1:21">
@@ -3299,16 +3369,19 @@
         <v>6</v>
       </c>
       <c r="F35" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G35" s="19">
         <v>1234567923</v>
       </c>
       <c r="H35" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I35" s="20">
         <v>10032</v>
+      </c>
+      <c r="J35" s="21">
+        <v>85032</v>
       </c>
     </row>
     <row r="36" ht="16.35" spans="1:21">
@@ -3322,18 +3395,20 @@
         <v>1</v>
       </c>
       <c r="F36" s="44" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G36" s="19">
         <v>1234567924</v>
       </c>
       <c r="H36" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I36" s="20">
         <v>10033</v>
       </c>
-      <c r="J36" s="32"/>
+      <c r="J36" s="21">
+        <v>85033</v>
+      </c>
       <c r="K36" s="32"/>
       <c r="L36" s="32"/>
       <c r="M36" s="32"/>
@@ -3353,18 +3428,20 @@
         <v>2</v>
       </c>
       <c r="F37" s="52" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G37" s="19">
         <v>1234567925</v>
       </c>
       <c r="H37" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I37" s="20">
         <v>10034</v>
       </c>
-      <c r="J37" s="21"/>
+      <c r="J37" s="21">
+        <v>85034</v>
+      </c>
       <c r="K37" s="21"/>
       <c r="L37" s="21"/>
       <c r="M37" s="21"/>
@@ -3384,18 +3461,20 @@
         <v>3</v>
       </c>
       <c r="F38" s="25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G38" s="19">
         <v>1234567926</v>
       </c>
       <c r="H38" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I38" s="20">
         <v>10035</v>
       </c>
-      <c r="J38" s="21"/>
+      <c r="J38" s="21">
+        <v>85035</v>
+      </c>
       <c r="K38" s="21"/>
       <c r="L38" s="21"/>
       <c r="M38" s="21"/>
@@ -3419,18 +3498,20 @@
         <v>4</v>
       </c>
       <c r="F39" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G39" s="19">
         <v>1234567927</v>
       </c>
       <c r="H39" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I39" s="20">
         <v>10036</v>
       </c>
-      <c r="J39" s="22"/>
+      <c r="J39" s="21">
+        <v>85036</v>
+      </c>
       <c r="K39" s="21"/>
       <c r="L39" s="21"/>
       <c r="M39" s="21"/>
@@ -3450,18 +3531,20 @@
         <v>5</v>
       </c>
       <c r="F40" s="34" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G40" s="19">
         <v>1234567928</v>
       </c>
       <c r="H40" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I40" s="20">
         <v>10037</v>
       </c>
-      <c r="J40" s="21"/>
+      <c r="J40" s="21">
+        <v>85037</v>
+      </c>
       <c r="K40" s="21"/>
       <c r="L40" s="21"/>
       <c r="M40" s="21"/>
@@ -3481,18 +3564,20 @@
         <v>6</v>
       </c>
       <c r="F41" s="34" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G41" s="19">
         <v>1234567929</v>
       </c>
       <c r="H41" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I41" s="20">
         <v>10038</v>
       </c>
-      <c r="J41" s="35"/>
+      <c r="J41" s="21">
+        <v>85038</v>
+      </c>
       <c r="K41" s="35"/>
       <c r="L41" s="35"/>
       <c r="M41" s="35"/>
@@ -3514,18 +3599,20 @@
         <v>1</v>
       </c>
       <c r="F42" s="44" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G42" s="19">
         <v>1234567930</v>
       </c>
       <c r="H42" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I42" s="20">
         <v>10039</v>
       </c>
-      <c r="J42" s="32"/>
+      <c r="J42" s="21">
+        <v>85039</v>
+      </c>
       <c r="K42" s="32"/>
       <c r="L42" s="32"/>
       <c r="M42" s="32"/>
@@ -3545,18 +3632,20 @@
         <v>2</v>
       </c>
       <c r="F43" s="50" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G43" s="19">
         <v>1234567931</v>
       </c>
       <c r="H43" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I43" s="20">
         <v>10040</v>
       </c>
-      <c r="J43" s="21"/>
+      <c r="J43" s="21">
+        <v>85040</v>
+      </c>
       <c r="K43" s="21"/>
       <c r="L43" s="21"/>
       <c r="M43" s="21"/>
@@ -3576,18 +3665,20 @@
         <v>3</v>
       </c>
       <c r="F44" s="58" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G44" s="19">
         <v>1234567932</v>
       </c>
       <c r="H44" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I44" s="20">
         <v>10041</v>
       </c>
-      <c r="J44" s="35"/>
+      <c r="J44" s="21">
+        <v>85041</v>
+      </c>
       <c r="K44" s="35"/>
       <c r="L44" s="35"/>
       <c r="M44" s="35"/>
@@ -3609,18 +3700,20 @@
         <v>1</v>
       </c>
       <c r="F45" s="37" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G45" s="19">
         <v>1234567933</v>
       </c>
       <c r="H45" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I45" s="20">
         <v>10042</v>
       </c>
-      <c r="J45" s="32"/>
+      <c r="J45" s="21">
+        <v>85042</v>
+      </c>
       <c r="K45" s="32"/>
       <c r="L45" s="32"/>
       <c r="M45" s="32"/>
@@ -3640,18 +3733,20 @@
         <v>2</v>
       </c>
       <c r="F46" s="59" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G46" s="19">
         <v>1234567934</v>
       </c>
       <c r="H46" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I46" s="20">
         <v>10043</v>
       </c>
-      <c r="J46" s="21"/>
+      <c r="J46" s="21">
+        <v>85043</v>
+      </c>
       <c r="K46" s="21"/>
       <c r="L46" s="21"/>
       <c r="M46" s="21"/>
@@ -3671,18 +3766,20 @@
         <v>3</v>
       </c>
       <c r="F47" s="44" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G47" s="19">
         <v>1234567935</v>
       </c>
       <c r="H47" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I47" s="20">
         <v>10044</v>
       </c>
-      <c r="J47" s="32"/>
+      <c r="J47" s="21">
+        <v>85044</v>
+      </c>
       <c r="K47" s="32"/>
       <c r="L47" s="32"/>
       <c r="M47" s="32"/>
@@ -3702,18 +3799,20 @@
         <v>4</v>
       </c>
       <c r="F48" s="60" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G48" s="19">
         <v>1234567936</v>
       </c>
       <c r="H48" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I48" s="20">
         <v>10045</v>
       </c>
-      <c r="J48" s="21"/>
+      <c r="J48" s="21">
+        <v>85045</v>
+      </c>
       <c r="K48" s="21"/>
       <c r="L48" s="21"/>
       <c r="M48" s="21"/>
@@ -3733,18 +3832,20 @@
         <v>5</v>
       </c>
       <c r="F49" s="38" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G49" s="19">
         <v>1234567937</v>
       </c>
       <c r="H49" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I49" s="20">
         <v>10046</v>
       </c>
-      <c r="J49" s="21"/>
+      <c r="J49" s="21">
+        <v>85046</v>
+      </c>
       <c r="K49" s="21"/>
       <c r="L49" s="21"/>
       <c r="M49" s="21"/>
@@ -3764,18 +3865,20 @@
         <v>6</v>
       </c>
       <c r="F50" s="40" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G50" s="19">
         <v>1234567938</v>
       </c>
       <c r="H50" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I50" s="20">
         <v>10047</v>
       </c>
-      <c r="J50" s="21"/>
+      <c r="J50" s="21">
+        <v>85047</v>
+      </c>
       <c r="K50" s="21"/>
       <c r="L50" s="21"/>
       <c r="M50" s="21"/>
@@ -3797,18 +3900,20 @@
         <v>1</v>
       </c>
       <c r="F51" s="34" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G51" s="19">
         <v>1234567939</v>
       </c>
       <c r="H51" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I51" s="20">
         <v>10048</v>
       </c>
-      <c r="J51" s="21"/>
+      <c r="J51" s="21">
+        <v>85048</v>
+      </c>
       <c r="K51" s="21"/>
       <c r="L51" s="21"/>
       <c r="M51" s="21"/>
@@ -3828,18 +3933,20 @@
         <v>2</v>
       </c>
       <c r="F52" s="61" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G52" s="19">
         <v>1234567940</v>
       </c>
       <c r="H52" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I52" s="20">
         <v>10049</v>
       </c>
-      <c r="J52" s="21"/>
+      <c r="J52" s="21">
+        <v>85049</v>
+      </c>
       <c r="K52" s="21"/>
       <c r="L52" s="21"/>
       <c r="M52" s="21"/>
@@ -3859,18 +3966,20 @@
         <v>3</v>
       </c>
       <c r="F53" s="25" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G53" s="19">
         <v>1234567941</v>
       </c>
       <c r="H53" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I53" s="20">
         <v>10050</v>
       </c>
-      <c r="J53" s="21"/>
+      <c r="J53" s="21">
+        <v>85050</v>
+      </c>
       <c r="K53" s="21"/>
       <c r="L53" s="21"/>
       <c r="M53" s="21"/>
@@ -3890,18 +3999,20 @@
         <v>4</v>
       </c>
       <c r="F54" s="59" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G54" s="19">
         <v>1234567942</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I54" s="20">
         <v>10051</v>
       </c>
-      <c r="J54" s="21"/>
+      <c r="J54" s="21">
+        <v>85051</v>
+      </c>
       <c r="K54" s="21"/>
       <c r="L54" s="21"/>
       <c r="M54" s="21"/>
@@ -3921,18 +4032,20 @@
         <v>5</v>
       </c>
       <c r="F55" s="40" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G55" s="19">
         <v>1234567943</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I55" s="20">
         <v>10052</v>
       </c>
-      <c r="J55" s="21"/>
+      <c r="J55" s="21">
+        <v>85052</v>
+      </c>
       <c r="K55" s="21"/>
       <c r="L55" s="21"/>
       <c r="M55" s="21"/>
@@ -3952,18 +4065,20 @@
         <v>6</v>
       </c>
       <c r="F56" s="38" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G56" s="19">
         <v>1234567944</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I56" s="20">
         <v>10053</v>
       </c>
-      <c r="J56" s="39"/>
+      <c r="J56" s="21">
+        <v>85053</v>
+      </c>
       <c r="K56" s="39"/>
       <c r="L56" s="39"/>
       <c r="M56" s="39"/>
@@ -3985,18 +4100,20 @@
         <v>1</v>
       </c>
       <c r="F57" s="56" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G57" s="19">
         <v>1234567945</v>
       </c>
       <c r="H57" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I57" s="20">
         <v>10054</v>
       </c>
-      <c r="J57" s="21"/>
+      <c r="J57" s="21">
+        <v>85054</v>
+      </c>
       <c r="K57" s="21"/>
       <c r="L57" s="21"/>
       <c r="M57" s="21"/>
@@ -4016,18 +4133,20 @@
         <v>2</v>
       </c>
       <c r="F58" s="62" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G58" s="19">
         <v>1234567946</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I58" s="20">
         <v>10055</v>
       </c>
-      <c r="J58" s="21"/>
+      <c r="J58" s="21">
+        <v>85055</v>
+      </c>
       <c r="K58" s="21"/>
       <c r="L58" s="21"/>
       <c r="M58" s="21"/>
@@ -4047,18 +4166,20 @@
         <v>3</v>
       </c>
       <c r="F59" s="34" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G59" s="19">
         <v>1234567947</v>
       </c>
       <c r="H59" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I59" s="20">
         <v>10056</v>
       </c>
-      <c r="J59" s="35"/>
+      <c r="J59" s="21">
+        <v>85056</v>
+      </c>
       <c r="K59" s="35"/>
       <c r="L59" s="35"/>
       <c r="M59" s="35"/>
@@ -4080,18 +4201,20 @@
         <v>1</v>
       </c>
       <c r="F60" s="41" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G60" s="19">
         <v>1234567948</v>
       </c>
       <c r="H60" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I60" s="20">
         <v>10057</v>
       </c>
-      <c r="J60" s="42"/>
+      <c r="J60" s="21">
+        <v>85057</v>
+      </c>
       <c r="K60" s="42"/>
       <c r="L60" s="42"/>
       <c r="M60" s="42"/>
@@ -4111,18 +4234,20 @@
         <v>2</v>
       </c>
       <c r="F61" s="34" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G61" s="19">
         <v>1234567949</v>
       </c>
       <c r="H61" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I61" s="20">
         <v>10058</v>
       </c>
-      <c r="J61" s="21"/>
+      <c r="J61" s="21">
+        <v>85058</v>
+      </c>
       <c r="K61" s="21"/>
       <c r="L61" s="21"/>
       <c r="M61" s="21"/>
@@ -4142,18 +4267,20 @@
         <v>3</v>
       </c>
       <c r="F62" s="34" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G62" s="19">
         <v>1234567950</v>
       </c>
       <c r="H62" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I62" s="20">
         <v>10059</v>
       </c>
-      <c r="J62" s="21"/>
+      <c r="J62" s="21">
+        <v>85059</v>
+      </c>
       <c r="K62" s="21"/>
       <c r="L62" s="21"/>
       <c r="M62" s="21"/>
@@ -4175,18 +4302,20 @@
         <v>1</v>
       </c>
       <c r="F63" s="37" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G63" s="19">
         <v>1234567951</v>
       </c>
       <c r="H63" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I63" s="20">
         <v>10060</v>
       </c>
-      <c r="J63" s="32"/>
+      <c r="J63" s="21">
+        <v>85060</v>
+      </c>
       <c r="K63" s="32"/>
       <c r="L63" s="32"/>
       <c r="M63" s="32"/>
@@ -4206,18 +4335,20 @@
         <v>2</v>
       </c>
       <c r="F64" s="52" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G64" s="19">
         <v>1234567952</v>
       </c>
       <c r="H64" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I64" s="20">
         <v>10061</v>
       </c>
-      <c r="J64" s="21"/>
+      <c r="J64" s="21">
+        <v>85061</v>
+      </c>
       <c r="K64" s="21"/>
       <c r="L64" s="21"/>
       <c r="M64" s="21"/>
@@ -4237,18 +4368,20 @@
         <v>3</v>
       </c>
       <c r="F65" s="52" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G65" s="19">
         <v>1234567953</v>
       </c>
       <c r="H65" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I65" s="20">
         <v>10062</v>
       </c>
-      <c r="J65" s="21"/>
+      <c r="J65" s="21">
+        <v>85062</v>
+      </c>
       <c r="K65" s="21"/>
       <c r="L65" s="21"/>
       <c r="M65" s="21"/>
@@ -4268,18 +4401,20 @@
         <v>4</v>
       </c>
       <c r="F66" s="25" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G66" s="19">
         <v>1234567954</v>
       </c>
       <c r="H66" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I66" s="20">
         <v>10063</v>
       </c>
-      <c r="J66" s="21"/>
+      <c r="J66" s="21">
+        <v>85063</v>
+      </c>
       <c r="K66" s="21"/>
       <c r="L66" s="21"/>
       <c r="M66" s="21"/>
@@ -4299,18 +4434,20 @@
         <v>5</v>
       </c>
       <c r="F67" s="64" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G67" s="19">
         <v>1234567955</v>
       </c>
       <c r="H67" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I67" s="20">
         <v>10064</v>
       </c>
-      <c r="J67" s="22"/>
+      <c r="J67" s="21">
+        <v>85064</v>
+      </c>
       <c r="K67" s="22"/>
       <c r="L67" s="22"/>
       <c r="M67" s="22"/>
@@ -4329,18 +4466,20 @@
         <v>6</v>
       </c>
       <c r="F68" s="65" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G68" s="19">
         <v>1234567956</v>
       </c>
       <c r="H68" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I68" s="20">
         <v>10065</v>
       </c>
-      <c r="J68" s="35"/>
+      <c r="J68" s="21">
+        <v>85065</v>
+      </c>
       <c r="K68" s="35"/>
       <c r="L68" s="35"/>
       <c r="M68" s="35"/>
@@ -4358,18 +4497,20 @@
       <c r="D69" s="24"/>
       <c r="E69" s="47"/>
       <c r="F69" s="37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G69" s="19">
         <v>1234567957</v>
       </c>
       <c r="H69" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I69" s="20">
         <v>10066</v>
       </c>
-      <c r="J69" s="32"/>
+      <c r="J69" s="21">
+        <v>85066</v>
+      </c>
       <c r="K69" s="32"/>
       <c r="L69" s="32"/>
       <c r="M69" s="32"/>
@@ -4391,18 +4532,20 @@
         <v>1</v>
       </c>
       <c r="F70" s="37" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G70" s="19">
         <v>1234567958</v>
       </c>
       <c r="H70" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I70" s="20">
         <v>10067</v>
       </c>
-      <c r="J70" s="32"/>
+      <c r="J70" s="21">
+        <v>85067</v>
+      </c>
       <c r="K70" s="32"/>
       <c r="L70" s="32"/>
       <c r="M70" s="32"/>
@@ -4422,18 +4565,20 @@
         <v>2</v>
       </c>
       <c r="F71" s="25" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G71" s="19">
         <v>1234567959</v>
       </c>
       <c r="H71" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I71" s="20">
         <v>10068</v>
       </c>
-      <c r="J71" s="21"/>
+      <c r="J71" s="21">
+        <v>85068</v>
+      </c>
       <c r="K71" s="21"/>
       <c r="L71" s="21"/>
       <c r="M71" s="21"/>
@@ -4453,18 +4598,20 @@
         <v>3</v>
       </c>
       <c r="F72" s="25" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G72" s="19">
         <v>1234567960</v>
       </c>
       <c r="H72" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I72" s="20">
         <v>10069</v>
       </c>
-      <c r="J72" s="21"/>
+      <c r="J72" s="21">
+        <v>85069</v>
+      </c>
       <c r="K72" s="21"/>
       <c r="L72" s="21"/>
       <c r="M72" s="21"/>
@@ -4484,18 +4631,20 @@
         <v>4</v>
       </c>
       <c r="F73" s="37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G73" s="19">
         <v>1234567961</v>
       </c>
       <c r="H73" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I73" s="20">
         <v>10070</v>
       </c>
-      <c r="J73" s="21"/>
+      <c r="J73" s="21">
+        <v>85070</v>
+      </c>
       <c r="K73" s="21"/>
       <c r="L73" s="21"/>
       <c r="M73" s="21"/>
@@ -4515,18 +4664,20 @@
         <v>5</v>
       </c>
       <c r="F74" s="37" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G74" s="19">
         <v>1234567962</v>
       </c>
       <c r="H74" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I74" s="20">
         <v>10071</v>
       </c>
-      <c r="J74" s="32"/>
+      <c r="J74" s="21">
+        <v>85071</v>
+      </c>
       <c r="K74" s="32"/>
       <c r="L74" s="32"/>
       <c r="M74" s="32"/>
@@ -4546,16 +4697,19 @@
         <v>6</v>
       </c>
       <c r="F75" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G75" s="19">
         <v>1234567963</v>
       </c>
       <c r="H75" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I75" s="20">
         <v>10072</v>
+      </c>
+      <c r="J75" s="21">
+        <v>85072</v>
       </c>
     </row>
     <row r="76" ht="16.35" spans="1:19">
@@ -4569,18 +4723,20 @@
         <v>1</v>
       </c>
       <c r="F76" s="37" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G76" s="19">
         <v>1234567964</v>
       </c>
       <c r="H76" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I76" s="20">
         <v>10073</v>
       </c>
-      <c r="J76" s="32"/>
+      <c r="J76" s="21">
+        <v>85073</v>
+      </c>
       <c r="K76" s="32"/>
       <c r="L76" s="32"/>
       <c r="M76" s="32"/>
@@ -4600,18 +4756,20 @@
         <v>2</v>
       </c>
       <c r="F77" s="25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G77" s="19">
         <v>1234567965</v>
       </c>
       <c r="H77" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I77" s="20">
         <v>10074</v>
       </c>
-      <c r="J77" s="21"/>
+      <c r="J77" s="21">
+        <v>85074</v>
+      </c>
       <c r="K77" s="21"/>
       <c r="L77" s="21"/>
       <c r="M77" s="21"/>
@@ -4631,18 +4789,20 @@
         <v>3</v>
       </c>
       <c r="F78" s="40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G78" s="19">
         <v>1234567966</v>
       </c>
       <c r="H78" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I78" s="20">
         <v>10075</v>
       </c>
-      <c r="J78" s="21"/>
+      <c r="J78" s="21">
+        <v>85075</v>
+      </c>
       <c r="K78" s="21"/>
       <c r="L78" s="21"/>
       <c r="M78" s="21"/>
@@ -4664,18 +4824,20 @@
         <v>1</v>
       </c>
       <c r="F79" s="66" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G79" s="19">
         <v>1234567967</v>
       </c>
       <c r="H79" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I79" s="20">
         <v>10076</v>
       </c>
-      <c r="J79" s="32"/>
+      <c r="J79" s="21">
+        <v>85076</v>
+      </c>
       <c r="K79" s="32"/>
       <c r="L79" s="32"/>
       <c r="M79" s="32"/>
@@ -4695,16 +4857,19 @@
         <v>2</v>
       </c>
       <c r="F80" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G80" s="19">
         <v>1234567968</v>
       </c>
       <c r="H80" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I80" s="20">
         <v>10077</v>
+      </c>
+      <c r="J80" s="21">
+        <v>85077</v>
       </c>
       <c r="O80" s="67"/>
       <c r="P80" s="32"/>
@@ -4718,18 +4883,20 @@
         <v>3</v>
       </c>
       <c r="F81" s="64" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G81" s="19">
         <v>1234567969</v>
       </c>
       <c r="H81" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I81" s="20">
         <v>10078</v>
       </c>
-      <c r="J81" s="21"/>
+      <c r="J81" s="21">
+        <v>85078</v>
+      </c>
       <c r="K81" s="21"/>
       <c r="L81" s="21"/>
       <c r="M81" s="21"/>
@@ -4749,18 +4916,20 @@
         <v>4</v>
       </c>
       <c r="F82" s="40" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G82" s="19">
         <v>1234567970</v>
       </c>
       <c r="H82" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I82" s="20">
         <v>10079</v>
       </c>
-      <c r="J82" s="21"/>
+      <c r="J82" s="21">
+        <v>85079</v>
+      </c>
       <c r="K82" s="21"/>
       <c r="L82" s="21"/>
       <c r="M82" s="21"/>
@@ -4780,18 +4949,20 @@
         <v>5</v>
       </c>
       <c r="F83" s="40" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G83" s="19">
         <v>1234567971</v>
       </c>
       <c r="H83" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I83" s="20">
         <v>10080</v>
       </c>
-      <c r="J83" s="21"/>
+      <c r="J83" s="21">
+        <v>85080</v>
+      </c>
       <c r="K83" s="21"/>
       <c r="L83" s="21"/>
       <c r="M83" s="21"/>
@@ -4811,18 +4982,20 @@
         <v>6</v>
       </c>
       <c r="F84" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G84" s="19">
         <v>1234567972</v>
       </c>
       <c r="H84" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I84" s="20">
         <v>10081</v>
       </c>
-      <c r="J84" s="69"/>
+      <c r="J84" s="21">
+        <v>85081</v>
+      </c>
       <c r="K84" s="69"/>
       <c r="L84" s="69"/>
       <c r="M84" s="69"/>
@@ -4844,18 +5017,20 @@
         <v>1</v>
       </c>
       <c r="F85" s="25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G85" s="19">
         <v>1234567973</v>
       </c>
       <c r="H85" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I85" s="20">
         <v>10082</v>
       </c>
-      <c r="J85" s="21"/>
+      <c r="J85" s="21">
+        <v>85082</v>
+      </c>
       <c r="K85" s="21"/>
       <c r="L85" s="21"/>
       <c r="M85" s="21"/>
@@ -4873,18 +5048,20 @@
       <c r="D86" s="24"/>
       <c r="E86" s="45"/>
       <c r="F86" s="40" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G86" s="19">
         <v>1234567974</v>
       </c>
       <c r="H86" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I86" s="20">
         <v>10083</v>
       </c>
-      <c r="J86" s="21"/>
+      <c r="J86" s="21">
+        <v>85083</v>
+      </c>
       <c r="K86" s="21"/>
       <c r="L86" s="21"/>
       <c r="M86" s="21"/>
@@ -4904,16 +5081,19 @@
         <v>2</v>
       </c>
       <c r="F87" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G87" s="19">
         <v>1234567975</v>
       </c>
       <c r="H87" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I87" s="20">
         <v>10084</v>
+      </c>
+      <c r="J87" s="21">
+        <v>85084</v>
       </c>
     </row>
     <row r="88" ht="17.1" spans="1:19">
@@ -4923,18 +5103,20 @@
       <c r="D88" s="24"/>
       <c r="E88" s="45"/>
       <c r="F88" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G88" s="19">
         <v>1234567976</v>
       </c>
       <c r="H88" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I88" s="20">
         <v>10085</v>
       </c>
-      <c r="J88" s="21"/>
+      <c r="J88" s="21">
+        <v>85085</v>
+      </c>
       <c r="K88" s="21"/>
       <c r="L88" s="21"/>
       <c r="M88" s="21"/>
@@ -4954,16 +5136,19 @@
         <v>3</v>
       </c>
       <c r="F89" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G89" s="19">
         <v>1234567977</v>
       </c>
       <c r="H89" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I89" s="20">
         <v>10086</v>
+      </c>
+      <c r="J89" s="21">
+        <v>85086</v>
       </c>
     </row>
     <row r="90" ht="17.1" spans="1:19">
@@ -4975,18 +5160,20 @@
         <v>4</v>
       </c>
       <c r="F90" s="56" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G90" s="19">
         <v>1234567978</v>
       </c>
       <c r="H90" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I90" s="20">
         <v>10087</v>
       </c>
-      <c r="J90" s="21"/>
+      <c r="J90" s="21">
+        <v>85087</v>
+      </c>
       <c r="K90" s="21"/>
       <c r="L90" s="21"/>
       <c r="M90" s="21"/>
@@ -5006,18 +5193,20 @@
         <v>5</v>
       </c>
       <c r="F91" s="59" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G91" s="19">
         <v>1234567979</v>
       </c>
       <c r="H91" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I91" s="20">
         <v>10088</v>
       </c>
-      <c r="J91" s="21"/>
+      <c r="J91" s="21">
+        <v>85088</v>
+      </c>
       <c r="K91" s="21"/>
       <c r="L91" s="21"/>
       <c r="M91" s="21"/>
@@ -5037,18 +5226,20 @@
         <v>6</v>
       </c>
       <c r="F92" s="43" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G92" s="19">
         <v>1234567980</v>
       </c>
       <c r="H92" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I92" s="20">
         <v>10089</v>
       </c>
-      <c r="J92" s="71"/>
+      <c r="J92" s="21">
+        <v>85089</v>
+      </c>
       <c r="K92" s="71"/>
       <c r="L92" s="71"/>
       <c r="M92" s="71"/>
@@ -5070,18 +5261,20 @@
         <v>1</v>
       </c>
       <c r="F93" s="73" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G93" s="19">
         <v>1234567981</v>
       </c>
       <c r="H93" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I93" s="20">
         <v>10090</v>
       </c>
-      <c r="J93" s="32"/>
+      <c r="J93" s="21">
+        <v>85090</v>
+      </c>
       <c r="K93" s="32"/>
       <c r="L93" s="32"/>
       <c r="M93" s="32"/>
@@ -5101,18 +5294,20 @@
         <v>2</v>
       </c>
       <c r="F94" s="25" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G94" s="19">
         <v>1234567982</v>
       </c>
       <c r="H94" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I94" s="20">
         <v>10091</v>
       </c>
-      <c r="J94" s="21"/>
+      <c r="J94" s="21">
+        <v>85091</v>
+      </c>
       <c r="K94" s="21"/>
       <c r="L94" s="21"/>
       <c r="M94" s="21"/>
@@ -5132,18 +5327,20 @@
         <v>3</v>
       </c>
       <c r="F95" s="43" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G95" s="19">
         <v>1234567983</v>
       </c>
       <c r="H95" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I95" s="20">
         <v>10092</v>
       </c>
-      <c r="J95" s="35"/>
+      <c r="J95" s="21">
+        <v>85092</v>
+      </c>
       <c r="K95" s="35"/>
       <c r="L95" s="35"/>
       <c r="M95" s="35"/>
@@ -5165,18 +5362,20 @@
         <v>1</v>
       </c>
       <c r="F96" s="37" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G96" s="19">
         <v>1234567984</v>
       </c>
       <c r="H96" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I96" s="20">
         <v>10093</v>
       </c>
-      <c r="J96" s="32"/>
+      <c r="J96" s="21">
+        <v>85093</v>
+      </c>
       <c r="K96" s="32"/>
       <c r="L96" s="32"/>
       <c r="M96" s="32"/>
@@ -5196,18 +5395,20 @@
         <v>2</v>
       </c>
       <c r="F97" s="40" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G97" s="19">
         <v>1234567985</v>
       </c>
       <c r="H97" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I97" s="20">
         <v>10094</v>
       </c>
-      <c r="J97" s="21"/>
+      <c r="J97" s="21">
+        <v>85094</v>
+      </c>
       <c r="K97" s="21"/>
       <c r="L97" s="21"/>
       <c r="M97" s="21"/>
@@ -5227,18 +5428,20 @@
         <v>3</v>
       </c>
       <c r="F98" s="40" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G98" s="19">
         <v>1234567986</v>
       </c>
       <c r="H98" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I98" s="20">
         <v>10095</v>
       </c>
-      <c r="J98" s="21"/>
+      <c r="J98" s="21">
+        <v>85095</v>
+      </c>
       <c r="K98" s="21"/>
       <c r="L98" s="21"/>
       <c r="M98" s="21"/>
@@ -5258,18 +5461,20 @@
         <v>4</v>
       </c>
       <c r="F99" s="40" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G99" s="19">
         <v>1234567987</v>
       </c>
       <c r="H99" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I99" s="20">
         <v>10096</v>
       </c>
-      <c r="J99" s="21"/>
+      <c r="J99" s="21">
+        <v>85096</v>
+      </c>
       <c r="K99" s="21"/>
       <c r="L99" s="21"/>
       <c r="M99" s="21"/>
@@ -5292,18 +5497,20 @@
         <v>5</v>
       </c>
       <c r="F100" s="75" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G100" s="19">
         <v>1234567988</v>
       </c>
       <c r="H100" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I100" s="20">
         <v>10097</v>
       </c>
-      <c r="J100" s="32"/>
+      <c r="J100" s="21">
+        <v>85097</v>
+      </c>
       <c r="K100" s="32"/>
       <c r="L100" s="32"/>
       <c r="M100" s="32"/>
@@ -5323,18 +5530,20 @@
         <v>6</v>
       </c>
       <c r="F101" s="64" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G101" s="19">
         <v>1234567989</v>
       </c>
       <c r="H101" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I101" s="20">
         <v>10098</v>
       </c>
-      <c r="J101" s="77"/>
+      <c r="J101" s="21">
+        <v>85098</v>
+      </c>
       <c r="K101" s="77"/>
       <c r="L101" s="77"/>
       <c r="M101" s="77"/>
@@ -5356,18 +5565,20 @@
         <v>1</v>
       </c>
       <c r="F102" s="37" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G102" s="19">
         <v>1234567990</v>
       </c>
       <c r="H102" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I102" s="20">
         <v>10099</v>
       </c>
-      <c r="J102" s="32"/>
+      <c r="J102" s="21">
+        <v>85099</v>
+      </c>
       <c r="K102" s="32"/>
       <c r="L102" s="32"/>
       <c r="M102" s="32"/>
@@ -5387,18 +5598,20 @@
         <v>2</v>
       </c>
       <c r="F103" s="25" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G103" s="19">
         <v>1234567991</v>
       </c>
       <c r="H103" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I103" s="20">
         <v>10100</v>
       </c>
-      <c r="J103" s="21"/>
+      <c r="J103" s="21">
+        <v>85100</v>
+      </c>
       <c r="K103" s="21"/>
       <c r="L103" s="21"/>
       <c r="M103" s="21"/>
@@ -5418,18 +5631,20 @@
         <v>3</v>
       </c>
       <c r="F104" s="40" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G104" s="19">
         <v>1234567992</v>
       </c>
       <c r="H104" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I104" s="20">
         <v>10101</v>
       </c>
-      <c r="J104" s="21"/>
+      <c r="J104" s="21">
+        <v>85101</v>
+      </c>
       <c r="K104" s="21"/>
       <c r="L104" s="21"/>
       <c r="M104" s="21"/>
@@ -5449,18 +5664,20 @@
         <v>4</v>
       </c>
       <c r="F105" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G105" s="19">
         <v>1234567993</v>
       </c>
       <c r="H105" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I105" s="20">
         <v>10102</v>
       </c>
-      <c r="J105" s="78"/>
+      <c r="J105" s="21">
+        <v>85102</v>
+      </c>
       <c r="K105" s="78"/>
       <c r="L105" s="78"/>
       <c r="M105" s="78"/>
@@ -5480,18 +5697,20 @@
         <v>5</v>
       </c>
       <c r="F106" s="40" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G106" s="19">
         <v>1234567994</v>
       </c>
       <c r="H106" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I106" s="20">
         <v>10103</v>
       </c>
-      <c r="J106" s="21"/>
+      <c r="J106" s="21">
+        <v>85103</v>
+      </c>
       <c r="K106" s="21"/>
       <c r="L106" s="21"/>
       <c r="M106" s="21"/>
@@ -5511,18 +5730,20 @@
         <v>6</v>
       </c>
       <c r="F107" s="64" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G107" s="19">
         <v>1234567995</v>
       </c>
       <c r="H107" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I107" s="20">
         <v>10104</v>
       </c>
-      <c r="J107" s="35"/>
+      <c r="J107" s="21">
+        <v>85104</v>
+      </c>
       <c r="K107" s="35"/>
       <c r="L107" s="35"/>
       <c r="M107" s="35"/>
@@ -5544,18 +5765,20 @@
         <v>1</v>
       </c>
       <c r="F108" s="37" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G108" s="19">
         <v>1234567996</v>
       </c>
       <c r="H108" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I108" s="20">
         <v>10105</v>
       </c>
-      <c r="J108" s="32"/>
+      <c r="J108" s="21">
+        <v>85105</v>
+      </c>
       <c r="K108" s="32"/>
       <c r="L108" s="32"/>
       <c r="M108" s="32"/>
@@ -5575,18 +5798,20 @@
         <v>2</v>
       </c>
       <c r="F109" s="38" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G109" s="19">
         <v>1234567997</v>
       </c>
       <c r="H109" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I109" s="20">
         <v>10106</v>
       </c>
-      <c r="J109" s="21"/>
+      <c r="J109" s="21">
+        <v>85106</v>
+      </c>
       <c r="K109" s="21"/>
       <c r="L109" s="21"/>
       <c r="M109" s="21"/>
@@ -5606,18 +5831,20 @@
         <v>3</v>
       </c>
       <c r="F110" s="62" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G110" s="19">
         <v>1234567998</v>
       </c>
       <c r="H110" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I110" s="20">
         <v>10107</v>
       </c>
-      <c r="J110" s="21"/>
+      <c r="J110" s="21">
+        <v>85107</v>
+      </c>
       <c r="K110" s="21"/>
       <c r="L110" s="21"/>
       <c r="M110" s="21"/>
@@ -5637,18 +5864,20 @@
         <v>4</v>
       </c>
       <c r="F111" s="49" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G111" s="19">
         <v>1234567999</v>
       </c>
       <c r="H111" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I111" s="20">
         <v>10108</v>
       </c>
-      <c r="J111" s="21"/>
+      <c r="J111" s="21">
+        <v>85108</v>
+      </c>
       <c r="K111" s="21"/>
       <c r="L111" s="21"/>
       <c r="M111" s="21"/>
@@ -5668,18 +5897,20 @@
         <v>5</v>
       </c>
       <c r="F112" s="64" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G112" s="19">
         <v>1234568000</v>
       </c>
       <c r="H112" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I112" s="20">
         <v>10109</v>
       </c>
-      <c r="J112" s="21"/>
+      <c r="J112" s="21">
+        <v>85109</v>
+      </c>
       <c r="K112" s="21"/>
       <c r="L112" s="21"/>
       <c r="M112" s="21"/>
@@ -5699,18 +5930,20 @@
         <v>6</v>
       </c>
       <c r="F113" s="52" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G113" s="19">
         <v>1234568001</v>
       </c>
       <c r="H113" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I113" s="20">
         <v>10110</v>
       </c>
-      <c r="J113" s="21"/>
+      <c r="J113" s="21">
+        <v>85110</v>
+      </c>
       <c r="K113" s="21"/>
       <c r="L113" s="21"/>
       <c r="M113" s="21"/>
@@ -5732,18 +5965,20 @@
         <v>1</v>
       </c>
       <c r="F114" s="48" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G114" s="19">
         <v>1234568002</v>
       </c>
       <c r="H114" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I114" s="20">
         <v>10111</v>
       </c>
-      <c r="J114" s="32"/>
+      <c r="J114" s="21">
+        <v>85111</v>
+      </c>
       <c r="K114" s="32"/>
       <c r="L114" s="32"/>
       <c r="M114" s="32"/>
@@ -5763,18 +5998,20 @@
         <v>2</v>
       </c>
       <c r="F115" s="82" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G115" s="19">
         <v>1234568003</v>
       </c>
       <c r="H115" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I115" s="20">
         <v>10112</v>
       </c>
-      <c r="J115" s="21"/>
+      <c r="J115" s="21">
+        <v>85112</v>
+      </c>
       <c r="K115" s="21"/>
       <c r="L115" s="21"/>
       <c r="M115" s="21"/>
@@ -5794,18 +6031,20 @@
         <v>3</v>
       </c>
       <c r="F116" s="40" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G116" s="19">
         <v>1234568004</v>
       </c>
       <c r="H116" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I116" s="20">
         <v>10113</v>
       </c>
-      <c r="J116" s="21"/>
+      <c r="J116" s="21">
+        <v>85113</v>
+      </c>
       <c r="K116" s="21"/>
       <c r="L116" s="21"/>
       <c r="M116" s="21"/>
@@ -5827,18 +6066,20 @@
         <v>1</v>
       </c>
       <c r="F117" s="37" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G117" s="19">
         <v>1234568005</v>
       </c>
       <c r="H117" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I117" s="20">
         <v>10114</v>
       </c>
-      <c r="J117" s="32"/>
+      <c r="J117" s="21">
+        <v>85114</v>
+      </c>
       <c r="K117" s="32"/>
       <c r="L117" s="32"/>
       <c r="M117" s="32"/>
@@ -5858,18 +6099,20 @@
         <v>2</v>
       </c>
       <c r="F118" s="59" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G118" s="19">
         <v>1234568006</v>
       </c>
       <c r="H118" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I118" s="20">
         <v>10115</v>
       </c>
-      <c r="J118" s="21"/>
+      <c r="J118" s="21">
+        <v>85115</v>
+      </c>
       <c r="K118" s="21"/>
       <c r="L118" s="21"/>
       <c r="M118" s="21"/>
@@ -5889,18 +6132,20 @@
         <v>3</v>
       </c>
       <c r="F119" s="53" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G119" s="19">
         <v>1234568007</v>
       </c>
       <c r="H119" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I119" s="20">
         <v>10116</v>
       </c>
-      <c r="J119" s="21"/>
+      <c r="J119" s="21">
+        <v>85116</v>
+      </c>
       <c r="K119" s="21"/>
       <c r="L119" s="21"/>
       <c r="M119" s="21"/>
@@ -5920,18 +6165,20 @@
         <v>4</v>
       </c>
       <c r="F120" s="83" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G120" s="19">
         <v>1234568008</v>
       </c>
       <c r="H120" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I120" s="20">
         <v>10117</v>
       </c>
-      <c r="J120" s="21"/>
+      <c r="J120" s="21">
+        <v>85117</v>
+      </c>
       <c r="K120" s="21"/>
       <c r="L120" s="21"/>
       <c r="M120" s="21"/>
@@ -5951,18 +6198,20 @@
         <v>5</v>
       </c>
       <c r="F121" s="38" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G121" s="19">
         <v>1234568009</v>
       </c>
       <c r="H121" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I121" s="20">
         <v>10118</v>
       </c>
-      <c r="J121" s="39"/>
+      <c r="J121" s="21">
+        <v>85118</v>
+      </c>
       <c r="K121" s="39"/>
       <c r="L121" s="39"/>
       <c r="M121" s="39"/>
@@ -5982,18 +6231,20 @@
         <v>6</v>
       </c>
       <c r="F122" s="34" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G122" s="19">
         <v>1234568010</v>
       </c>
       <c r="H122" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I122" s="20">
         <v>10119</v>
       </c>
-      <c r="J122" s="35"/>
+      <c r="J122" s="21">
+        <v>85119</v>
+      </c>
       <c r="K122" s="35"/>
       <c r="L122" s="35"/>
       <c r="M122" s="35"/>
@@ -6015,18 +6266,20 @@
         <v>1</v>
       </c>
       <c r="F123" s="85" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G123" s="19">
         <v>1234568011</v>
       </c>
       <c r="H123" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I123" s="20">
         <v>10120</v>
       </c>
-      <c r="J123" s="32"/>
+      <c r="J123" s="21">
+        <v>85120</v>
+      </c>
       <c r="K123" s="32"/>
       <c r="L123" s="32"/>
       <c r="M123" s="32"/>
@@ -6046,18 +6299,20 @@
         <v>2</v>
       </c>
       <c r="F124" s="25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G124" s="19">
         <v>1234568012</v>
       </c>
       <c r="H124" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I124" s="20">
         <v>10121</v>
       </c>
-      <c r="J124" s="21"/>
+      <c r="J124" s="21">
+        <v>85121</v>
+      </c>
       <c r="K124" s="21"/>
       <c r="L124" s="21"/>
       <c r="M124" s="21"/>
@@ -6077,18 +6332,20 @@
         <v>3</v>
       </c>
       <c r="F125" s="25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G125" s="19">
         <v>1234568013</v>
       </c>
       <c r="H125" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I125" s="20">
         <v>10122</v>
       </c>
-      <c r="J125" s="21"/>
+      <c r="J125" s="21">
+        <v>85122</v>
+      </c>
       <c r="K125" s="21"/>
       <c r="L125" s="21"/>
       <c r="M125" s="21"/>
@@ -6108,18 +6365,20 @@
         <v>4</v>
       </c>
       <c r="F126" s="38" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G126" s="19">
         <v>1234568014</v>
       </c>
       <c r="H126" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I126" s="20">
         <v>10123</v>
       </c>
-      <c r="J126" s="21"/>
+      <c r="J126" s="21">
+        <v>85123</v>
+      </c>
       <c r="K126" s="21"/>
       <c r="L126" s="21"/>
       <c r="M126" s="21"/>
@@ -6139,18 +6398,20 @@
         <v>5</v>
       </c>
       <c r="F127" s="52" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G127" s="19">
         <v>1234568015</v>
       </c>
       <c r="H127" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I127" s="20">
         <v>10124</v>
       </c>
-      <c r="J127" s="21"/>
+      <c r="J127" s="21">
+        <v>85124</v>
+      </c>
       <c r="K127" s="21"/>
       <c r="L127" s="21"/>
       <c r="M127" s="21"/>
@@ -6170,18 +6431,20 @@
         <v>6</v>
       </c>
       <c r="F128" s="65" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G128" s="19">
         <v>1234568016</v>
       </c>
       <c r="H128" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I128" s="20">
         <v>10125</v>
       </c>
-      <c r="J128" s="35"/>
+      <c r="J128" s="21">
+        <v>85125</v>
+      </c>
       <c r="K128" s="35"/>
       <c r="L128" s="35"/>
       <c r="M128" s="35"/>
@@ -6203,18 +6466,20 @@
         <v>1</v>
       </c>
       <c r="F129" s="66" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G129" s="19">
         <v>1234568017</v>
       </c>
       <c r="H129" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I129" s="20">
         <v>10126</v>
       </c>
-      <c r="J129" s="42"/>
+      <c r="J129" s="21">
+        <v>85126</v>
+      </c>
       <c r="K129" s="22"/>
       <c r="L129" s="42"/>
       <c r="M129" s="22"/>
@@ -6234,18 +6499,20 @@
         <v>2</v>
       </c>
       <c r="F130" s="37" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G130" s="19">
         <v>1234568018</v>
       </c>
       <c r="H130" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I130" s="20">
         <v>10127</v>
       </c>
-      <c r="J130" s="21"/>
+      <c r="J130" s="21">
+        <v>85127</v>
+      </c>
       <c r="K130" s="21"/>
       <c r="L130" s="21"/>
       <c r="M130" s="21"/>
@@ -6265,18 +6532,20 @@
         <v>3</v>
       </c>
       <c r="F131" s="75" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G131" s="19">
         <v>1234568019</v>
       </c>
       <c r="H131" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I131" s="20">
         <v>10128</v>
       </c>
-      <c r="J131" s="39"/>
+      <c r="J131" s="21">
+        <v>85128</v>
+      </c>
       <c r="K131" s="39"/>
       <c r="L131" s="39"/>
       <c r="M131" s="39"/>
@@ -6296,16 +6565,19 @@
         <v>4</v>
       </c>
       <c r="F132" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G132" s="19">
         <v>1234568020</v>
       </c>
       <c r="H132" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I132" s="20">
         <v>10129</v>
+      </c>
+      <c r="J132" s="21">
+        <v>85129</v>
       </c>
     </row>
     <row r="133" ht="17.1" spans="1:19">
@@ -6317,18 +6589,20 @@
         <v>5</v>
       </c>
       <c r="F133" s="41" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G133" s="19">
         <v>1234568021</v>
       </c>
       <c r="H133" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I133" s="20">
         <v>10130</v>
       </c>
-      <c r="J133" s="21"/>
+      <c r="J133" s="21">
+        <v>85130</v>
+      </c>
       <c r="K133" s="21"/>
       <c r="L133" s="21"/>
       <c r="M133" s="21"/>
@@ -6348,18 +6622,20 @@
         <v>6</v>
       </c>
       <c r="F134" s="88" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G134" s="19">
         <v>1234568022</v>
       </c>
       <c r="H134" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I134" s="20">
         <v>10131</v>
       </c>
-      <c r="J134" s="39"/>
+      <c r="J134" s="21">
+        <v>85131</v>
+      </c>
       <c r="K134" s="39"/>
       <c r="L134" s="39"/>
       <c r="M134" s="39"/>
@@ -6381,18 +6657,20 @@
         <v>1</v>
       </c>
       <c r="F135" s="40" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G135" s="19">
         <v>1234568023</v>
       </c>
       <c r="H135" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I135" s="20">
         <v>10132</v>
       </c>
-      <c r="J135" s="21"/>
+      <c r="J135" s="21">
+        <v>85132</v>
+      </c>
       <c r="K135" s="21"/>
       <c r="L135" s="21"/>
       <c r="M135" s="21"/>
@@ -6412,18 +6690,20 @@
         <v>2</v>
       </c>
       <c r="F136" s="89" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G136" s="19">
         <v>1234568024</v>
       </c>
       <c r="H136" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I136" s="20">
         <v>10133</v>
       </c>
-      <c r="J136" s="32"/>
+      <c r="J136" s="21">
+        <v>85133</v>
+      </c>
       <c r="K136" s="32"/>
       <c r="L136" s="32"/>
       <c r="M136" s="32"/>
@@ -6443,18 +6723,20 @@
         <v>3</v>
       </c>
       <c r="F137" s="25" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G137" s="19">
         <v>1234568025</v>
       </c>
       <c r="H137" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I137" s="20">
         <v>10134</v>
       </c>
-      <c r="J137" s="21"/>
+      <c r="J137" s="21">
+        <v>85134</v>
+      </c>
       <c r="K137" s="21"/>
       <c r="L137" s="21"/>
       <c r="M137" s="21"/>
@@ -6474,18 +6756,20 @@
         <v>4</v>
       </c>
       <c r="F138" s="75" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G138" s="19">
         <v>1234568026</v>
       </c>
       <c r="H138" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I138" s="20">
         <v>10135</v>
       </c>
-      <c r="J138" s="21"/>
+      <c r="J138" s="21">
+        <v>85135</v>
+      </c>
       <c r="K138" s="21"/>
       <c r="L138" s="21"/>
       <c r="M138" s="21"/>
@@ -6505,18 +6789,20 @@
         <v>5</v>
       </c>
       <c r="F139" s="40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G139" s="19">
         <v>1234568027</v>
       </c>
       <c r="H139" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I139" s="20">
         <v>10136</v>
       </c>
-      <c r="J139" s="21"/>
+      <c r="J139" s="21">
+        <v>85136</v>
+      </c>
       <c r="K139" s="21"/>
       <c r="L139" s="21"/>
       <c r="M139" s="21"/>
@@ -6536,18 +6822,20 @@
         <v>6</v>
       </c>
       <c r="F140" s="62" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G140" s="19">
         <v>1234568028</v>
       </c>
       <c r="H140" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I140" s="20">
         <v>10137</v>
       </c>
-      <c r="J140" s="21"/>
+      <c r="J140" s="21">
+        <v>85137</v>
+      </c>
       <c r="K140" s="21"/>
       <c r="L140" s="21"/>
       <c r="M140" s="21"/>
@@ -6569,18 +6857,20 @@
         <v>1</v>
       </c>
       <c r="F141" s="90" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G141" s="19">
         <v>1234568029</v>
       </c>
       <c r="H141" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I141" s="20">
         <v>10138</v>
       </c>
-      <c r="J141" s="21"/>
+      <c r="J141" s="21">
+        <v>85138</v>
+      </c>
       <c r="K141" s="21"/>
       <c r="L141" s="21"/>
       <c r="M141" s="21"/>
@@ -6600,18 +6890,20 @@
         <v>2</v>
       </c>
       <c r="F142" s="91" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G142" s="19">
         <v>1234568030</v>
       </c>
       <c r="H142" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I142" s="20">
         <v>10139</v>
       </c>
-      <c r="J142" s="21"/>
+      <c r="J142" s="21">
+        <v>85139</v>
+      </c>
       <c r="K142" s="21"/>
       <c r="L142" s="21"/>
       <c r="M142" s="21"/>
@@ -6631,18 +6923,20 @@
         <v>3</v>
       </c>
       <c r="F143" s="25" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G143" s="19">
         <v>1234568031</v>
       </c>
       <c r="H143" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I143" s="20">
         <v>10140</v>
       </c>
-      <c r="J143" s="21"/>
+      <c r="J143" s="21">
+        <v>85140</v>
+      </c>
       <c r="K143" s="21"/>
       <c r="L143" s="21"/>
       <c r="M143" s="21"/>
@@ -6662,18 +6956,20 @@
         <v>4</v>
       </c>
       <c r="F144" s="37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G144" s="19">
         <v>1234568032</v>
       </c>
       <c r="H144" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I144" s="20">
         <v>10141</v>
       </c>
-      <c r="J144" s="32"/>
+      <c r="J144" s="21">
+        <v>85141</v>
+      </c>
       <c r="K144" s="32"/>
       <c r="L144" s="32"/>
       <c r="M144" s="32"/>
@@ -6693,18 +6989,20 @@
         <v>5</v>
       </c>
       <c r="F145" s="52" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G145" s="19">
         <v>1234568033</v>
       </c>
       <c r="H145" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I145" s="20">
         <v>10142</v>
       </c>
-      <c r="J145" s="21"/>
+      <c r="J145" s="21">
+        <v>85142</v>
+      </c>
       <c r="K145" s="21"/>
       <c r="L145" s="21"/>
       <c r="M145" s="21"/>
@@ -6724,18 +7022,20 @@
         <v>6</v>
       </c>
       <c r="F146" s="92" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G146" s="19">
         <v>1234568034</v>
       </c>
       <c r="H146" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I146" s="20">
         <v>10143</v>
       </c>
-      <c r="J146" s="35"/>
+      <c r="J146" s="21">
+        <v>85143</v>
+      </c>
       <c r="K146" s="35"/>
       <c r="L146" s="35"/>
       <c r="M146" s="35"/>
@@ -6757,18 +7057,20 @@
         <v>1</v>
       </c>
       <c r="F147" s="37" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G147" s="19">
         <v>1234568035</v>
       </c>
       <c r="H147" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I147" s="20">
         <v>10144</v>
       </c>
-      <c r="J147" s="32"/>
+      <c r="J147" s="21">
+        <v>85144</v>
+      </c>
       <c r="K147" s="32"/>
       <c r="L147" s="32"/>
       <c r="M147" s="32"/>
@@ -6788,18 +7090,20 @@
         <v>2</v>
       </c>
       <c r="F148" s="93" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G148" s="19">
         <v>1234568036</v>
       </c>
       <c r="H148" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I148" s="20">
         <v>10145</v>
       </c>
-      <c r="J148" s="21"/>
+      <c r="J148" s="21">
+        <v>85145</v>
+      </c>
       <c r="K148" s="21"/>
       <c r="L148" s="21"/>
       <c r="M148" s="21"/>
@@ -6810,7 +7114,7 @@
       <c r="R148" s="23"/>
       <c r="S148" s="21"/>
       <c r="U148" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="149" spans="1:21">
@@ -6822,18 +7126,20 @@
         <v>3</v>
       </c>
       <c r="F149" s="40" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G149" s="19">
         <v>1234568037</v>
       </c>
       <c r="H149" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I149" s="20">
         <v>10146</v>
       </c>
-      <c r="J149" s="21"/>
+      <c r="J149" s="21">
+        <v>85146</v>
+      </c>
       <c r="K149" s="21"/>
       <c r="L149" s="21"/>
       <c r="M149" s="21"/>
@@ -6853,18 +7159,20 @@
         <v>4</v>
       </c>
       <c r="F150" s="40" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G150" s="19">
         <v>1234568038</v>
       </c>
       <c r="H150" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I150" s="20">
         <v>10147</v>
       </c>
-      <c r="J150" s="32"/>
+      <c r="J150" s="21">
+        <v>85147</v>
+      </c>
       <c r="K150" s="32"/>
       <c r="L150" s="32"/>
       <c r="M150" s="32"/>
@@ -6884,18 +7192,20 @@
         <v>5</v>
       </c>
       <c r="F151" s="92" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G151" s="19">
         <v>1234568039</v>
       </c>
       <c r="H151" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I151" s="20">
         <v>10148</v>
       </c>
-      <c r="J151" s="21"/>
+      <c r="J151" s="21">
+        <v>85148</v>
+      </c>
       <c r="K151" s="21"/>
       <c r="L151" s="21"/>
       <c r="M151" s="21"/>
@@ -6915,18 +7225,20 @@
         <v>6</v>
       </c>
       <c r="F152" s="94" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G152" s="19">
         <v>1234568040</v>
       </c>
       <c r="H152" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I152" s="20">
         <v>10149</v>
       </c>
-      <c r="J152" s="21"/>
+      <c r="J152" s="21">
+        <v>85149</v>
+      </c>
       <c r="K152" s="21"/>
       <c r="L152" s="21"/>
       <c r="M152" s="21"/>
@@ -6948,18 +7260,20 @@
         <v>1</v>
       </c>
       <c r="F153" s="37" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G153" s="19">
         <v>1234568041</v>
       </c>
       <c r="H153" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I153" s="20">
         <v>10150</v>
       </c>
-      <c r="J153" s="32"/>
+      <c r="J153" s="21">
+        <v>85150</v>
+      </c>
       <c r="K153" s="32"/>
       <c r="L153" s="32"/>
       <c r="M153" s="32"/>
@@ -6979,18 +7293,20 @@
         <v>2</v>
       </c>
       <c r="F154" s="34" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G154" s="19">
         <v>1234568042</v>
       </c>
       <c r="H154" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I154" s="20">
         <v>10151</v>
       </c>
-      <c r="J154" s="21"/>
+      <c r="J154" s="21">
+        <v>85151</v>
+      </c>
       <c r="K154" s="21"/>
       <c r="L154" s="21"/>
       <c r="M154" s="21"/>
@@ -7010,18 +7326,20 @@
         <v>3</v>
       </c>
       <c r="F155" s="50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G155" s="19">
         <v>1234568043</v>
       </c>
       <c r="H155" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I155" s="20">
         <v>10152</v>
       </c>
-      <c r="J155" s="21"/>
+      <c r="J155" s="21">
+        <v>85152</v>
+      </c>
       <c r="K155" s="21"/>
       <c r="L155" s="21"/>
       <c r="M155" s="21"/>
@@ -7041,18 +7359,20 @@
         <v>4</v>
       </c>
       <c r="F156" s="25" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G156" s="19">
         <v>1234568044</v>
       </c>
       <c r="H156" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I156" s="20">
         <v>10153</v>
       </c>
-      <c r="J156" s="21"/>
+      <c r="J156" s="21">
+        <v>85153</v>
+      </c>
       <c r="K156" s="21"/>
       <c r="L156" s="21"/>
       <c r="M156" s="21"/>
@@ -7072,18 +7392,20 @@
         <v>5</v>
       </c>
       <c r="F157" s="34" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G157" s="19">
         <v>1234568045</v>
       </c>
       <c r="H157" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I157" s="20">
         <v>10154</v>
       </c>
-      <c r="J157" s="21"/>
+      <c r="J157" s="21">
+        <v>85154</v>
+      </c>
       <c r="K157" s="21"/>
       <c r="L157" s="21"/>
       <c r="M157" s="21"/>
@@ -7103,18 +7425,20 @@
         <v>6</v>
       </c>
       <c r="F158" s="38" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G158" s="19">
         <v>1234568046</v>
       </c>
       <c r="H158" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I158" s="20">
         <v>10155</v>
       </c>
-      <c r="J158" s="39"/>
+      <c r="J158" s="21">
+        <v>85155</v>
+      </c>
       <c r="K158" s="39"/>
       <c r="L158" s="39"/>
       <c r="M158" s="39"/>
@@ -7136,18 +7460,20 @@
         <v>1</v>
       </c>
       <c r="F159" s="64" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G159" s="19">
         <v>1234568047</v>
       </c>
       <c r="H159" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I159" s="20">
         <v>10156</v>
       </c>
-      <c r="J159" s="21"/>
+      <c r="J159" s="21">
+        <v>85156</v>
+      </c>
       <c r="K159" s="21"/>
       <c r="L159" s="21"/>
       <c r="M159" s="21"/>
@@ -7167,18 +7493,20 @@
         <v>2</v>
       </c>
       <c r="F160" s="38" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G160" s="19">
         <v>1234568048</v>
       </c>
       <c r="H160" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I160" s="20">
         <v>10157</v>
       </c>
-      <c r="J160" s="21"/>
+      <c r="J160" s="21">
+        <v>85157</v>
+      </c>
       <c r="K160" s="21"/>
       <c r="L160" s="21"/>
       <c r="M160" s="21"/>
@@ -7198,18 +7526,20 @@
         <v>3</v>
       </c>
       <c r="F161" s="52" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G161" s="19">
         <v>1234568049</v>
       </c>
       <c r="H161" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I161" s="20">
         <v>10158</v>
       </c>
-      <c r="J161" s="21"/>
+      <c r="J161" s="21">
+        <v>85158</v>
+      </c>
       <c r="K161" s="21"/>
       <c r="L161" s="21"/>
       <c r="M161" s="21"/>
@@ -7229,18 +7559,20 @@
         <v>4</v>
       </c>
       <c r="F162" s="52" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G162" s="19">
         <v>1234568050</v>
       </c>
       <c r="H162" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I162" s="20">
         <v>10159</v>
       </c>
-      <c r="J162" s="21"/>
+      <c r="J162" s="21">
+        <v>85159</v>
+      </c>
       <c r="K162" s="21"/>
       <c r="L162" s="21"/>
       <c r="M162" s="21"/>
@@ -7260,18 +7592,20 @@
         <v>5</v>
       </c>
       <c r="F163" s="22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G163" s="19">
         <v>1234568051</v>
       </c>
       <c r="H163" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I163" s="20">
         <v>10160</v>
       </c>
-      <c r="J163" s="22"/>
+      <c r="J163" s="21">
+        <v>85160</v>
+      </c>
       <c r="K163" s="22"/>
       <c r="L163" s="22"/>
       <c r="M163" s="22"/>
@@ -7291,18 +7625,20 @@
         <v>6</v>
       </c>
       <c r="F164" s="34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G164" s="19">
         <v>1234568052</v>
       </c>
       <c r="H164" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I164" s="20">
         <v>10161</v>
       </c>
-      <c r="J164" s="21"/>
+      <c r="J164" s="21">
+        <v>85161</v>
+      </c>
       <c r="K164" s="21"/>
       <c r="L164" s="21"/>
       <c r="M164" s="21"/>
@@ -7324,18 +7660,20 @@
         <v>1</v>
       </c>
       <c r="F165" s="40" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G165" s="19">
         <v>1234568053</v>
       </c>
       <c r="H165" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I165" s="20">
         <v>10162</v>
       </c>
-      <c r="J165" s="21"/>
+      <c r="J165" s="21">
+        <v>85162</v>
+      </c>
       <c r="K165" s="21"/>
       <c r="L165" s="21"/>
       <c r="M165" s="21"/>
@@ -7355,18 +7693,20 @@
         <v>2</v>
       </c>
       <c r="F166" s="40" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G166" s="19">
         <v>1234568054</v>
       </c>
       <c r="H166" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I166" s="20">
         <v>10163</v>
       </c>
-      <c r="J166" s="21"/>
+      <c r="J166" s="21">
+        <v>85163</v>
+      </c>
       <c r="K166" s="21"/>
       <c r="L166" s="21"/>
       <c r="M166" s="21"/>
@@ -7386,18 +7726,20 @@
         <v>3</v>
       </c>
       <c r="F167" s="25" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G167" s="19">
         <v>1234568055</v>
       </c>
       <c r="H167" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I167" s="20">
         <v>10164</v>
       </c>
-      <c r="J167" s="21"/>
+      <c r="J167" s="21">
+        <v>85164</v>
+      </c>
       <c r="K167" s="21"/>
       <c r="L167" s="21"/>
       <c r="M167" s="21"/>
@@ -7417,18 +7759,20 @@
         <v>4</v>
       </c>
       <c r="F168" s="61" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G168" s="19">
         <v>1234568056</v>
       </c>
       <c r="H168" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I168" s="20">
         <v>10165</v>
       </c>
-      <c r="J168" s="21"/>
+      <c r="J168" s="21">
+        <v>85165</v>
+      </c>
       <c r="K168" s="21"/>
       <c r="L168" s="21"/>
       <c r="M168" s="21"/>
@@ -7448,18 +7792,20 @@
         <v>5</v>
       </c>
       <c r="F169" s="52" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G169" s="19">
         <v>1234568057</v>
       </c>
       <c r="H169" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I169" s="20">
         <v>10166</v>
       </c>
-      <c r="J169" s="21"/>
+      <c r="J169" s="21">
+        <v>85166</v>
+      </c>
       <c r="K169" s="21"/>
       <c r="L169" s="21"/>
       <c r="M169" s="21"/>
@@ -7479,18 +7825,20 @@
         <v>6</v>
       </c>
       <c r="F170" s="34" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G170" s="19">
         <v>1234568058</v>
       </c>
       <c r="H170" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I170" s="20">
         <v>10167</v>
       </c>
-      <c r="J170" s="35"/>
+      <c r="J170" s="21">
+        <v>85167</v>
+      </c>
       <c r="K170" s="35"/>
       <c r="L170" s="35"/>
       <c r="M170" s="35"/>
@@ -7512,18 +7860,20 @@
         <v>1</v>
       </c>
       <c r="F171" s="37" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G171" s="19">
         <v>1234568059</v>
       </c>
       <c r="H171" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I171" s="20">
         <v>10168</v>
       </c>
-      <c r="J171" s="32"/>
+      <c r="J171" s="21">
+        <v>85168</v>
+      </c>
       <c r="K171" s="32"/>
       <c r="L171" s="32"/>
       <c r="M171" s="32"/>
@@ -7543,18 +7893,20 @@
         <v>2</v>
       </c>
       <c r="F172" s="25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G172" s="19">
         <v>1234568060</v>
       </c>
       <c r="H172" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I172" s="20">
         <v>10169</v>
       </c>
-      <c r="J172" s="21"/>
+      <c r="J172" s="21">
+        <v>85169</v>
+      </c>
       <c r="K172" s="21"/>
       <c r="L172" s="21"/>
       <c r="M172" s="21"/>
@@ -7574,18 +7926,20 @@
         <v>3</v>
       </c>
       <c r="F173" s="95" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G173" s="19">
         <v>1234568061</v>
       </c>
       <c r="H173" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I173" s="20">
         <v>10170</v>
       </c>
-      <c r="J173" s="21"/>
+      <c r="J173" s="21">
+        <v>85170</v>
+      </c>
       <c r="K173" s="21"/>
       <c r="L173" s="21"/>
       <c r="M173" s="21"/>
@@ -7605,18 +7959,20 @@
         <v>4</v>
       </c>
       <c r="F174" s="65" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G174" s="19">
         <v>1234568062</v>
       </c>
       <c r="H174" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I174" s="20">
         <v>10171</v>
       </c>
-      <c r="J174" s="21"/>
+      <c r="J174" s="21">
+        <v>85171</v>
+      </c>
       <c r="K174" s="21"/>
       <c r="L174" s="21"/>
       <c r="M174" s="21"/>
@@ -7636,18 +7992,20 @@
         <v>5</v>
       </c>
       <c r="F175" s="40" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G175" s="19">
         <v>1234568063</v>
       </c>
       <c r="H175" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I175" s="20">
         <v>10172</v>
       </c>
-      <c r="J175" s="21"/>
+      <c r="J175" s="21">
+        <v>85172</v>
+      </c>
       <c r="K175" s="21"/>
       <c r="L175" s="21"/>
       <c r="M175" s="21"/>
@@ -7667,18 +8025,20 @@
         <v>6</v>
       </c>
       <c r="F176" s="96" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G176" s="19">
         <v>1234568064</v>
       </c>
       <c r="H176" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I176" s="20">
         <v>10173</v>
       </c>
-      <c r="J176" s="35"/>
+      <c r="J176" s="21">
+        <v>85173</v>
+      </c>
       <c r="K176" s="35"/>
       <c r="L176" s="35"/>
       <c r="M176" s="35"/>
@@ -7700,18 +8060,20 @@
         <v>1</v>
       </c>
       <c r="F177" s="85" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G177" s="19">
         <v>1234568065</v>
       </c>
       <c r="H177" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I177" s="20">
         <v>10174</v>
       </c>
-      <c r="J177" s="32"/>
+      <c r="J177" s="21">
+        <v>85174</v>
+      </c>
       <c r="K177" s="32"/>
       <c r="L177" s="21"/>
       <c r="M177" s="21"/>
@@ -7731,18 +8093,20 @@
         <v>2</v>
       </c>
       <c r="F178" s="62" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G178" s="19">
         <v>1234568066</v>
       </c>
       <c r="H178" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I178" s="20">
         <v>10175</v>
       </c>
-      <c r="J178" s="39"/>
+      <c r="J178" s="21">
+        <v>85175</v>
+      </c>
       <c r="K178" s="39"/>
       <c r="L178" s="39"/>
       <c r="M178" s="39"/>
@@ -7762,18 +8126,20 @@
         <v>3</v>
       </c>
       <c r="F179" s="37" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G179" s="19">
         <v>1234568067</v>
       </c>
       <c r="H179" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I179" s="20">
         <v>10176</v>
       </c>
-      <c r="J179" s="21"/>
+      <c r="J179" s="21">
+        <v>85176</v>
+      </c>
       <c r="K179" s="21"/>
       <c r="L179" s="21"/>
       <c r="M179" s="21"/>
@@ -7795,18 +8161,20 @@
         <v>1</v>
       </c>
       <c r="F180" s="37" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G180" s="19">
         <v>1234568068</v>
       </c>
       <c r="H180" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I180" s="20">
         <v>10177</v>
       </c>
-      <c r="J180" s="32"/>
+      <c r="J180" s="21">
+        <v>85177</v>
+      </c>
       <c r="K180" s="32"/>
       <c r="L180" s="32"/>
       <c r="M180" s="32"/>
@@ -7826,16 +8194,19 @@
         <v>2</v>
       </c>
       <c r="F181" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G181" s="19">
         <v>1234568069</v>
       </c>
       <c r="H181" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I181" s="20">
         <v>10178</v>
+      </c>
+      <c r="J181" s="21">
+        <v>85178</v>
       </c>
       <c r="O181" s="67"/>
       <c r="P181" s="32"/>
@@ -7849,16 +8220,19 @@
         <v>3</v>
       </c>
       <c r="F182" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G182" s="19">
         <v>1234568070</v>
       </c>
       <c r="H182" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I182" s="20">
         <v>10179</v>
+      </c>
+      <c r="J182" s="21">
+        <v>85179</v>
       </c>
       <c r="O182" s="67"/>
       <c r="P182" s="32"/>
@@ -7872,18 +8246,20 @@
         <v>4</v>
       </c>
       <c r="F183" s="98" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G183" s="19">
         <v>1234568071</v>
       </c>
       <c r="H183" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I183" s="20">
         <v>10180</v>
       </c>
-      <c r="J183" s="21"/>
+      <c r="J183" s="21">
+        <v>85180</v>
+      </c>
       <c r="K183" s="21"/>
       <c r="L183" s="21"/>
       <c r="M183" s="21"/>
@@ -7903,18 +8279,20 @@
         <v>5</v>
       </c>
       <c r="F184" s="98" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G184" s="19">
         <v>1234568072</v>
       </c>
       <c r="H184" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I184" s="20">
         <v>10181</v>
       </c>
-      <c r="J184" s="21"/>
+      <c r="J184" s="21">
+        <v>85181</v>
+      </c>
       <c r="K184" s="21"/>
       <c r="L184" s="21"/>
       <c r="M184" s="21"/>
@@ -7934,18 +8312,20 @@
         <v>6</v>
       </c>
       <c r="F185" s="99" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G185" s="19">
         <v>1234568073</v>
       </c>
       <c r="H185" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I185" s="20">
         <v>10182</v>
       </c>
-      <c r="J185" s="21"/>
+      <c r="J185" s="21">
+        <v>85182</v>
+      </c>
       <c r="K185" s="21"/>
       <c r="L185" s="21"/>
       <c r="M185" s="21"/>
@@ -7967,18 +8347,20 @@
         <v>1</v>
       </c>
       <c r="F186" s="85" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G186" s="19">
         <v>1234568074</v>
       </c>
       <c r="H186" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I186" s="20">
         <v>10183</v>
       </c>
-      <c r="J186" s="32"/>
+      <c r="J186" s="21">
+        <v>85183</v>
+      </c>
       <c r="K186" s="32"/>
       <c r="L186" s="32"/>
       <c r="M186" s="32"/>
@@ -7998,18 +8380,20 @@
         <v>2</v>
       </c>
       <c r="F187" s="25" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G187" s="19">
         <v>1234568075</v>
       </c>
       <c r="H187" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I187" s="20">
         <v>10184</v>
       </c>
-      <c r="J187" s="21"/>
+      <c r="J187" s="21">
+        <v>85184</v>
+      </c>
       <c r="K187" s="21"/>
       <c r="L187" s="21"/>
       <c r="M187" s="21"/>
@@ -8029,18 +8413,20 @@
         <v>3</v>
       </c>
       <c r="F188" s="40" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G188" s="19">
         <v>1234568076</v>
       </c>
       <c r="H188" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I188" s="20">
         <v>10185</v>
       </c>
-      <c r="J188" s="21"/>
+      <c r="J188" s="21">
+        <v>85185</v>
+      </c>
       <c r="K188" s="21"/>
       <c r="L188" s="21"/>
       <c r="M188" s="21"/>
@@ -8060,16 +8446,19 @@
         <v>4</v>
       </c>
       <c r="F189" s="54" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G189" s="19">
         <v>1234568077</v>
       </c>
       <c r="H189" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I189" s="20">
         <v>10186</v>
+      </c>
+      <c r="J189" s="21">
+        <v>85186</v>
       </c>
     </row>
     <row r="190" ht="16.35" spans="1:20">
@@ -8081,18 +8470,20 @@
         <v>5</v>
       </c>
       <c r="F190" s="40" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G190" s="19">
         <v>1234568078</v>
       </c>
       <c r="H190" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I190" s="20">
         <v>10187</v>
       </c>
-      <c r="J190" s="32"/>
+      <c r="J190" s="21">
+        <v>85187</v>
+      </c>
       <c r="K190" s="32"/>
       <c r="L190" s="32"/>
       <c r="M190" s="32"/>
@@ -8112,18 +8503,20 @@
         <v>6</v>
       </c>
       <c r="F191" s="56" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G191" s="19">
         <v>1234568079</v>
       </c>
       <c r="H191" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I191" s="20">
         <v>10188</v>
       </c>
-      <c r="J191" s="21"/>
+      <c r="J191" s="21">
+        <v>85188</v>
+      </c>
       <c r="K191" s="21"/>
       <c r="L191" s="21"/>
       <c r="M191" s="21"/>
@@ -8146,18 +8539,20 @@
         <v>1</v>
       </c>
       <c r="F192" s="40" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G192" s="19">
         <v>1234568080</v>
       </c>
       <c r="H192" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I192" s="20">
         <v>10189</v>
       </c>
-      <c r="J192" s="21"/>
+      <c r="J192" s="21">
+        <v>85189</v>
+      </c>
       <c r="K192" s="21"/>
       <c r="L192" s="21"/>
       <c r="M192" s="21"/>
@@ -8177,18 +8572,20 @@
         <v>2</v>
       </c>
       <c r="F193" s="101" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G193" s="19">
         <v>1234568081</v>
       </c>
       <c r="H193" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I193" s="20">
         <v>10190</v>
       </c>
-      <c r="J193" s="21"/>
+      <c r="J193" s="21">
+        <v>85190</v>
+      </c>
       <c r="K193" s="21"/>
       <c r="L193" s="21"/>
       <c r="M193" s="21"/>
@@ -8208,18 +8605,20 @@
         <v>3</v>
       </c>
       <c r="F194" s="101" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G194" s="19">
         <v>1234568082</v>
       </c>
       <c r="H194" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I194" s="20">
         <v>10191</v>
       </c>
-      <c r="J194" s="21"/>
+      <c r="J194" s="21">
+        <v>85191</v>
+      </c>
       <c r="K194" s="21"/>
       <c r="L194" s="21"/>
       <c r="M194" s="21"/>
@@ -8239,18 +8638,20 @@
         <v>4</v>
       </c>
       <c r="F195" s="101" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G195" s="19">
         <v>1234568083</v>
       </c>
       <c r="H195" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I195" s="20">
         <v>10192</v>
       </c>
-      <c r="J195" s="21"/>
+      <c r="J195" s="21">
+        <v>85192</v>
+      </c>
       <c r="K195" s="21"/>
       <c r="L195" s="21"/>
       <c r="M195" s="21"/>
@@ -8270,18 +8671,20 @@
         <v>5</v>
       </c>
       <c r="F196" s="101" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G196" s="19">
         <v>1234568084</v>
       </c>
       <c r="H196" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I196" s="20">
         <v>10193</v>
       </c>
-      <c r="J196" s="21"/>
+      <c r="J196" s="21">
+        <v>85193</v>
+      </c>
       <c r="K196" s="21"/>
       <c r="L196" s="21"/>
       <c r="M196" s="21"/>
@@ -8301,18 +8704,20 @@
         <v>6</v>
       </c>
       <c r="F197" s="38" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G197" s="19">
         <v>1234568085</v>
       </c>
       <c r="H197" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I197" s="20">
         <v>10194</v>
       </c>
-      <c r="J197" s="35"/>
+      <c r="J197" s="21">
+        <v>85194</v>
+      </c>
       <c r="K197" s="35"/>
       <c r="L197" s="35"/>
       <c r="M197" s="35"/>
@@ -8334,18 +8739,20 @@
         <v>1</v>
       </c>
       <c r="F198" s="40" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G198" s="19">
         <v>1234568086</v>
       </c>
       <c r="H198" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I198" s="20">
         <v>10195</v>
       </c>
-      <c r="J198" s="32"/>
+      <c r="J198" s="21">
+        <v>85195</v>
+      </c>
       <c r="K198" s="32"/>
       <c r="L198" s="42"/>
       <c r="M198" s="32"/>
@@ -8365,18 +8772,20 @@
         <v>2</v>
       </c>
       <c r="F199" s="40" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G199" s="19">
         <v>1234568087</v>
       </c>
       <c r="H199" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I199" s="20">
         <v>10196</v>
       </c>
-      <c r="J199" s="21"/>
+      <c r="J199" s="21">
+        <v>85196</v>
+      </c>
       <c r="K199" s="21"/>
       <c r="L199" s="21"/>
       <c r="M199" s="21"/>
@@ -8396,18 +8805,20 @@
         <v>3</v>
       </c>
       <c r="F200" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G200" s="19">
         <v>1234568088</v>
       </c>
       <c r="H200" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I200" s="20">
         <v>10197</v>
       </c>
-      <c r="J200" s="21"/>
+      <c r="J200" s="21">
+        <v>85197</v>
+      </c>
       <c r="K200" s="21"/>
       <c r="L200" s="21"/>
       <c r="M200" s="21"/>
@@ -8427,18 +8838,20 @@
         <v>4</v>
       </c>
       <c r="F201" s="25" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G201" s="19">
         <v>1234568089</v>
       </c>
       <c r="H201" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I201" s="20">
         <v>10198</v>
       </c>
-      <c r="J201" s="21"/>
+      <c r="J201" s="21">
+        <v>85198</v>
+      </c>
       <c r="K201" s="21"/>
       <c r="L201" s="21"/>
       <c r="M201" s="21"/>
@@ -8458,18 +8871,20 @@
         <v>5</v>
       </c>
       <c r="F202" s="40" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G202" s="19">
         <v>1234568090</v>
       </c>
       <c r="H202" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I202" s="20">
         <v>10199</v>
       </c>
-      <c r="J202" s="21"/>
+      <c r="J202" s="21">
+        <v>85199</v>
+      </c>
       <c r="K202" s="21"/>
       <c r="L202" s="21"/>
       <c r="M202" s="21"/>
@@ -8489,18 +8904,20 @@
         <v>6</v>
       </c>
       <c r="F203" s="64" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G203" s="19">
         <v>1234568091</v>
       </c>
       <c r="H203" s="18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I203" s="20">
         <v>10200</v>
       </c>
-      <c r="J203" s="102"/>
+      <c r="J203" s="21">
+        <v>85200</v>
+      </c>
       <c r="K203" s="102"/>
       <c r="L203" s="102"/>
       <c r="M203" s="102"/>

</xml_diff>

<commit_message>
Update Excel student data
</commit_message>
<xml_diff>
--- a/Fees Details 2024-25.xlsx
+++ b/Fees Details 2024-25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HIMANSHU\hostel-management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D310BA04-7035-4375-BCFD-FDD1BB90F950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E13120FF-75D8-4FDE-87F3-6E4C905812C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="298">
   <si>
     <t>ROOMS</t>
   </si>
@@ -1110,12 +1110,63 @@
   <si>
     <t>vacate</t>
   </si>
+  <si>
+    <t>DORM</t>
+  </si>
+  <si>
+    <t>Kavish Navin Joshi</t>
+  </si>
+  <si>
+    <t>Vansh Kishor Jain</t>
+  </si>
+  <si>
+    <t>Laksh Tejraj Gogad</t>
+  </si>
+  <si>
+    <t>Akshay Anil Jain</t>
+  </si>
+  <si>
+    <t>Ayush Nitin Sharma</t>
+  </si>
+  <si>
+    <t>Pratham Santoshkumar Nahata</t>
+  </si>
+  <si>
+    <t>Sankalp Sheetalkumar Jain</t>
+  </si>
+  <si>
+    <t>Gaurang Milind Sharma</t>
+  </si>
+  <si>
+    <t>Veer Anand Sethi</t>
+  </si>
+  <si>
+    <t>Tanish Vikas Kochar</t>
+  </si>
+  <si>
+    <t>Param Shailesh Jain</t>
+  </si>
+  <si>
+    <t>Vatsal Rahul Achaliya</t>
+  </si>
+  <si>
+    <t>Bhavesh Ratimohan Modi</t>
+  </si>
+  <si>
+    <t>Yug Tushar Jain</t>
+  </si>
+  <si>
+    <t>MP</t>
+  </si>
+  <si>
+    <t>Maharashtra</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1166,6 +1217,18 @@
       <name val="Kokila"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Kokila"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1175,7 +1238,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1253,11 +1316,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1304,8 +1391,29 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1581,7 +1689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D1:J208"/>
+  <dimension ref="D1:J268"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="6" max="6" width="20.21875" customWidth="1"/>
@@ -6189,21 +6297,1034 @@
       <c r="J207" s="19"/>
     </row>
     <row r="208" spans="4:10" ht="19.2">
-      <c r="D208" s="7">
+      <c r="D208" s="23">
         <v>317</v>
       </c>
-      <c r="E208" s="14">
+      <c r="E208" s="24">
         <v>6</v>
       </c>
-      <c r="F208" s="18" t="s">
+      <c r="F208" s="25" t="s">
         <v>280</v>
       </c>
-      <c r="G208" s="19"/>
-      <c r="H208" s="19"/>
-      <c r="I208" s="19"/>
-      <c r="J208" s="19"/>
+      <c r="G208" s="26"/>
+      <c r="H208" s="26"/>
+      <c r="I208" s="26"/>
+      <c r="J208" s="26"/>
+    </row>
+    <row r="209" spans="4:10" ht="19.2">
+      <c r="D209" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E209" s="27">
+        <v>1</v>
+      </c>
+      <c r="F209" s="19" t="s">
+        <v>282</v>
+      </c>
+      <c r="G209" s="20">
+        <v>8889310551</v>
+      </c>
+      <c r="H209" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="I209" s="22">
+        <v>0</v>
+      </c>
+      <c r="J209" s="22">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="210" spans="4:10" ht="19.2">
+      <c r="D210" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E210" s="27">
+        <v>2</v>
+      </c>
+      <c r="F210" s="19" t="s">
+        <v>283</v>
+      </c>
+      <c r="G210" s="21">
+        <v>9421614398</v>
+      </c>
+      <c r="H210" s="21" t="s">
+        <v>297</v>
+      </c>
+      <c r="I210" s="22">
+        <v>3500</v>
+      </c>
+      <c r="J210" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="4:10" ht="19.2">
+      <c r="D211" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E211" s="27">
+        <v>3</v>
+      </c>
+      <c r="F211" s="19" t="s">
+        <v>284</v>
+      </c>
+      <c r="G211" s="21">
+        <v>9423193271</v>
+      </c>
+      <c r="H211" s="21" t="s">
+        <v>297</v>
+      </c>
+      <c r="I211" s="22">
+        <v>7000</v>
+      </c>
+      <c r="J211" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="4:10" ht="19.2">
+      <c r="D212" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E212" s="27">
+        <v>4</v>
+      </c>
+      <c r="F212" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="G212" s="21">
+        <v>9423918667</v>
+      </c>
+      <c r="H212" s="21" t="s">
+        <v>297</v>
+      </c>
+      <c r="I212" s="22">
+        <v>7000</v>
+      </c>
+      <c r="J212" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" spans="4:10" ht="19.2">
+      <c r="D213" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E213" s="27">
+        <v>5</v>
+      </c>
+      <c r="F213" s="19" t="s">
+        <v>286</v>
+      </c>
+      <c r="G213" s="21">
+        <v>9545516001</v>
+      </c>
+      <c r="H213" s="21" t="s">
+        <v>297</v>
+      </c>
+      <c r="I213" s="22">
+        <v>9000</v>
+      </c>
+      <c r="J213" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" spans="4:10" ht="19.2">
+      <c r="D214" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E214" s="27">
+        <v>6</v>
+      </c>
+      <c r="F214" s="19" t="s">
+        <v>287</v>
+      </c>
+      <c r="G214" s="20">
+        <v>9689839096</v>
+      </c>
+      <c r="H214" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="I214" s="22">
+        <v>7000</v>
+      </c>
+      <c r="J214" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215" spans="4:10" ht="19.2">
+      <c r="D215" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E215" s="27">
+        <v>7</v>
+      </c>
+      <c r="F215" s="19" t="s">
+        <v>288</v>
+      </c>
+      <c r="G215" s="20">
+        <v>9424070113</v>
+      </c>
+      <c r="H215" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="I215" s="22">
+        <v>27000</v>
+      </c>
+      <c r="J215" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216" spans="4:10" ht="19.2">
+      <c r="D216" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E216" s="27">
+        <v>8</v>
+      </c>
+      <c r="F216" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="G216" s="20">
+        <v>8208718482</v>
+      </c>
+      <c r="H216" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="I216" s="22">
+        <v>28000</v>
+      </c>
+      <c r="J216" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217" spans="4:10" ht="19.2">
+      <c r="D217" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E217" s="27">
+        <v>9</v>
+      </c>
+      <c r="F217" s="19" t="s">
+        <v>290</v>
+      </c>
+      <c r="G217" s="20">
+        <v>9322434650</v>
+      </c>
+      <c r="H217" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="I217" s="22">
+        <v>20000</v>
+      </c>
+      <c r="J217" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="4:10" ht="19.2">
+      <c r="D218" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E218" s="27">
+        <v>10</v>
+      </c>
+      <c r="F218" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="G218" s="20">
+        <v>9604379567</v>
+      </c>
+      <c r="H218" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="I218" s="22">
+        <v>15000</v>
+      </c>
+      <c r="J218" s="22">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="219" spans="4:10" ht="19.2">
+      <c r="D219" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E219" s="27">
+        <v>11</v>
+      </c>
+      <c r="F219" s="19" t="s">
+        <v>292</v>
+      </c>
+      <c r="G219" s="20">
+        <v>9421443513</v>
+      </c>
+      <c r="H219" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="I219" s="22">
+        <v>12000</v>
+      </c>
+      <c r="J219" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220" spans="4:10" ht="19.2">
+      <c r="D220" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E220" s="27">
+        <v>12</v>
+      </c>
+      <c r="F220" s="19" t="s">
+        <v>293</v>
+      </c>
+      <c r="G220" s="20">
+        <v>9850984144</v>
+      </c>
+      <c r="H220" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="I220" s="22">
+        <v>0</v>
+      </c>
+      <c r="J220" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221" spans="4:10" ht="19.2">
+      <c r="D221" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E221" s="27">
+        <v>13</v>
+      </c>
+      <c r="F221" s="19" t="s">
+        <v>294</v>
+      </c>
+      <c r="G221" s="20">
+        <v>7387938800</v>
+      </c>
+      <c r="H221" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="I221" s="22">
+        <v>12000</v>
+      </c>
+      <c r="J221" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222" spans="4:10" ht="19.2">
+      <c r="D222" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E222" s="27">
+        <v>14</v>
+      </c>
+      <c r="F222" s="19" t="s">
+        <v>295</v>
+      </c>
+      <c r="G222" s="20">
+        <v>7773902888</v>
+      </c>
+      <c r="H222" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="I222" s="22">
+        <v>10000</v>
+      </c>
+      <c r="J222" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223" spans="4:10" ht="19.2">
+      <c r="D223" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E223" s="27">
+        <v>15</v>
+      </c>
+      <c r="F223" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G223" s="19"/>
+      <c r="H223" s="19"/>
+      <c r="I223" s="19"/>
+      <c r="J223" s="19"/>
+    </row>
+    <row r="224" spans="4:10" ht="19.2">
+      <c r="D224" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E224" s="27">
+        <v>16</v>
+      </c>
+      <c r="F224" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G224" s="19"/>
+      <c r="H224" s="19"/>
+      <c r="I224" s="19"/>
+      <c r="J224" s="19"/>
+    </row>
+    <row r="225" spans="4:10" ht="19.2">
+      <c r="D225" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E225" s="27">
+        <v>17</v>
+      </c>
+      <c r="F225" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G225" s="19"/>
+      <c r="H225" s="19"/>
+      <c r="I225" s="19"/>
+      <c r="J225" s="19"/>
+    </row>
+    <row r="226" spans="4:10" ht="19.2">
+      <c r="D226" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E226" s="27">
+        <v>18</v>
+      </c>
+      <c r="F226" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G226" s="19"/>
+      <c r="H226" s="19"/>
+      <c r="I226" s="19"/>
+      <c r="J226" s="19"/>
+    </row>
+    <row r="227" spans="4:10" ht="19.2">
+      <c r="D227" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E227" s="27">
+        <v>19</v>
+      </c>
+      <c r="F227" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G227" s="19"/>
+      <c r="H227" s="19"/>
+      <c r="I227" s="19"/>
+      <c r="J227" s="19"/>
+    </row>
+    <row r="228" spans="4:10" ht="19.2">
+      <c r="D228" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E228" s="27">
+        <v>20</v>
+      </c>
+      <c r="F228" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G228" s="19"/>
+      <c r="H228" s="19"/>
+      <c r="I228" s="19"/>
+      <c r="J228" s="19"/>
+    </row>
+    <row r="229" spans="4:10" ht="19.2">
+      <c r="D229" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E229" s="27">
+        <v>21</v>
+      </c>
+      <c r="F229" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G229" s="19"/>
+      <c r="H229" s="19"/>
+      <c r="I229" s="19"/>
+      <c r="J229" s="19"/>
+    </row>
+    <row r="230" spans="4:10" ht="19.2">
+      <c r="D230" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E230" s="27">
+        <v>22</v>
+      </c>
+      <c r="F230" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G230" s="19"/>
+      <c r="H230" s="19"/>
+      <c r="I230" s="19"/>
+      <c r="J230" s="19"/>
+    </row>
+    <row r="231" spans="4:10" ht="19.2">
+      <c r="D231" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E231" s="27">
+        <v>23</v>
+      </c>
+      <c r="F231" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G231" s="19"/>
+      <c r="H231" s="19"/>
+      <c r="I231" s="19"/>
+      <c r="J231" s="19"/>
+    </row>
+    <row r="232" spans="4:10" ht="19.2">
+      <c r="D232" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E232" s="27">
+        <v>24</v>
+      </c>
+      <c r="F232" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G232" s="19"/>
+      <c r="H232" s="19"/>
+      <c r="I232" s="19"/>
+      <c r="J232" s="19"/>
+    </row>
+    <row r="233" spans="4:10" ht="19.2">
+      <c r="D233" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E233" s="27">
+        <v>25</v>
+      </c>
+      <c r="F233" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G233" s="19"/>
+      <c r="H233" s="19"/>
+      <c r="I233" s="19"/>
+      <c r="J233" s="19"/>
+    </row>
+    <row r="234" spans="4:10" ht="19.2">
+      <c r="D234" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E234" s="27">
+        <v>26</v>
+      </c>
+      <c r="F234" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G234" s="19"/>
+      <c r="H234" s="19"/>
+      <c r="I234" s="19"/>
+      <c r="J234" s="19"/>
+    </row>
+    <row r="235" spans="4:10" ht="19.2">
+      <c r="D235" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E235" s="27">
+        <v>27</v>
+      </c>
+      <c r="F235" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G235" s="19"/>
+      <c r="H235" s="19"/>
+      <c r="I235" s="19"/>
+      <c r="J235" s="19"/>
+    </row>
+    <row r="236" spans="4:10" ht="19.2">
+      <c r="D236" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E236" s="27">
+        <v>28</v>
+      </c>
+      <c r="F236" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G236" s="19"/>
+      <c r="H236" s="19"/>
+      <c r="I236" s="19"/>
+      <c r="J236" s="19"/>
+    </row>
+    <row r="237" spans="4:10" ht="19.2">
+      <c r="D237" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E237" s="27">
+        <v>29</v>
+      </c>
+      <c r="F237" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G237" s="19"/>
+      <c r="H237" s="19"/>
+      <c r="I237" s="19"/>
+      <c r="J237" s="19"/>
+    </row>
+    <row r="238" spans="4:10" ht="19.2">
+      <c r="D238" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E238" s="27">
+        <v>30</v>
+      </c>
+      <c r="F238" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G238" s="19"/>
+      <c r="H238" s="19"/>
+      <c r="I238" s="19"/>
+      <c r="J238" s="19"/>
+    </row>
+    <row r="239" spans="4:10" ht="19.2">
+      <c r="D239" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E239" s="27">
+        <v>31</v>
+      </c>
+      <c r="F239" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G239" s="19"/>
+      <c r="H239" s="19"/>
+      <c r="I239" s="19"/>
+      <c r="J239" s="19"/>
+    </row>
+    <row r="240" spans="4:10" ht="19.2">
+      <c r="D240" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E240" s="27">
+        <v>32</v>
+      </c>
+      <c r="F240" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G240" s="19"/>
+      <c r="H240" s="19"/>
+      <c r="I240" s="19"/>
+      <c r="J240" s="19"/>
+    </row>
+    <row r="241" spans="4:10" ht="19.2">
+      <c r="D241" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E241" s="27">
+        <v>33</v>
+      </c>
+      <c r="F241" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G241" s="19"/>
+      <c r="H241" s="19"/>
+      <c r="I241" s="19"/>
+      <c r="J241" s="19"/>
+    </row>
+    <row r="242" spans="4:10" ht="19.2">
+      <c r="D242" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E242" s="27">
+        <v>34</v>
+      </c>
+      <c r="F242" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G242" s="19"/>
+      <c r="H242" s="19"/>
+      <c r="I242" s="19"/>
+      <c r="J242" s="19"/>
+    </row>
+    <row r="243" spans="4:10" ht="19.2">
+      <c r="D243" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E243" s="27">
+        <v>35</v>
+      </c>
+      <c r="F243" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G243" s="19"/>
+      <c r="H243" s="19"/>
+      <c r="I243" s="19"/>
+      <c r="J243" s="19"/>
+    </row>
+    <row r="244" spans="4:10" ht="19.2">
+      <c r="D244" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E244" s="27">
+        <v>36</v>
+      </c>
+      <c r="F244" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G244" s="19"/>
+      <c r="H244" s="19"/>
+      <c r="I244" s="19"/>
+      <c r="J244" s="19"/>
+    </row>
+    <row r="245" spans="4:10" ht="19.2">
+      <c r="D245" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E245" s="27">
+        <v>37</v>
+      </c>
+      <c r="F245" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G245" s="19"/>
+      <c r="H245" s="19"/>
+      <c r="I245" s="19"/>
+      <c r="J245" s="19"/>
+    </row>
+    <row r="246" spans="4:10" ht="19.2">
+      <c r="D246" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E246" s="27">
+        <v>38</v>
+      </c>
+      <c r="F246" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G246" s="19"/>
+      <c r="H246" s="19"/>
+      <c r="I246" s="19"/>
+      <c r="J246" s="19"/>
+    </row>
+    <row r="247" spans="4:10" ht="19.2">
+      <c r="D247" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E247" s="27">
+        <v>39</v>
+      </c>
+      <c r="F247" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G247" s="19"/>
+      <c r="H247" s="19"/>
+      <c r="I247" s="19"/>
+      <c r="J247" s="19"/>
+    </row>
+    <row r="248" spans="4:10" ht="19.2">
+      <c r="D248" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E248" s="27">
+        <v>40</v>
+      </c>
+      <c r="F248" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G248" s="19"/>
+      <c r="H248" s="19"/>
+      <c r="I248" s="19"/>
+      <c r="J248" s="19"/>
+    </row>
+    <row r="249" spans="4:10" ht="19.2">
+      <c r="D249" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E249" s="27">
+        <v>41</v>
+      </c>
+      <c r="F249" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G249" s="19"/>
+      <c r="H249" s="19"/>
+      <c r="I249" s="19"/>
+      <c r="J249" s="19"/>
+    </row>
+    <row r="250" spans="4:10" ht="19.2">
+      <c r="D250" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E250" s="27">
+        <v>42</v>
+      </c>
+      <c r="F250" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G250" s="19"/>
+      <c r="H250" s="19"/>
+      <c r="I250" s="19"/>
+      <c r="J250" s="19"/>
+    </row>
+    <row r="251" spans="4:10" ht="19.2">
+      <c r="D251" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E251" s="27">
+        <v>43</v>
+      </c>
+      <c r="F251" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G251" s="19"/>
+      <c r="H251" s="19"/>
+      <c r="I251" s="19"/>
+      <c r="J251" s="19"/>
+    </row>
+    <row r="252" spans="4:10" ht="19.2">
+      <c r="D252" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E252" s="27">
+        <v>44</v>
+      </c>
+      <c r="F252" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G252" s="19"/>
+      <c r="H252" s="19"/>
+      <c r="I252" s="19"/>
+      <c r="J252" s="19"/>
+    </row>
+    <row r="253" spans="4:10" ht="19.2">
+      <c r="D253" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E253" s="27">
+        <v>45</v>
+      </c>
+      <c r="F253" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G253" s="19"/>
+      <c r="H253" s="19"/>
+      <c r="I253" s="19"/>
+      <c r="J253" s="19"/>
+    </row>
+    <row r="254" spans="4:10" ht="19.2">
+      <c r="D254" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E254" s="27">
+        <v>46</v>
+      </c>
+      <c r="F254" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G254" s="19"/>
+      <c r="H254" s="19"/>
+      <c r="I254" s="19"/>
+      <c r="J254" s="19"/>
+    </row>
+    <row r="255" spans="4:10" ht="19.2">
+      <c r="D255" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E255" s="27">
+        <v>47</v>
+      </c>
+      <c r="F255" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G255" s="19"/>
+      <c r="H255" s="19"/>
+      <c r="I255" s="19"/>
+      <c r="J255" s="19"/>
+    </row>
+    <row r="256" spans="4:10" ht="19.2">
+      <c r="D256" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E256" s="27">
+        <v>48</v>
+      </c>
+      <c r="F256" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G256" s="19"/>
+      <c r="H256" s="19"/>
+      <c r="I256" s="19"/>
+      <c r="J256" s="19"/>
+    </row>
+    <row r="257" spans="4:10" ht="19.2">
+      <c r="D257" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E257" s="27">
+        <v>49</v>
+      </c>
+      <c r="F257" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G257" s="19"/>
+      <c r="H257" s="19"/>
+      <c r="I257" s="19"/>
+      <c r="J257" s="19"/>
+    </row>
+    <row r="258" spans="4:10" ht="19.2">
+      <c r="D258" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E258" s="27">
+        <v>50</v>
+      </c>
+      <c r="F258" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G258" s="19"/>
+      <c r="H258" s="19"/>
+      <c r="I258" s="19"/>
+      <c r="J258" s="19"/>
+    </row>
+    <row r="259" spans="4:10" ht="19.2">
+      <c r="D259" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E259" s="27">
+        <v>51</v>
+      </c>
+      <c r="F259" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G259" s="19"/>
+      <c r="H259" s="19"/>
+      <c r="I259" s="19"/>
+      <c r="J259" s="19"/>
+    </row>
+    <row r="260" spans="4:10" ht="19.2">
+      <c r="D260" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E260" s="27">
+        <v>52</v>
+      </c>
+      <c r="F260" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G260" s="19"/>
+      <c r="H260" s="19"/>
+      <c r="I260" s="19"/>
+      <c r="J260" s="19"/>
+    </row>
+    <row r="261" spans="4:10" ht="19.2">
+      <c r="D261" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E261" s="27">
+        <v>53</v>
+      </c>
+      <c r="F261" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G261" s="19"/>
+      <c r="H261" s="19"/>
+      <c r="I261" s="19"/>
+      <c r="J261" s="19"/>
+    </row>
+    <row r="262" spans="4:10" ht="19.2">
+      <c r="D262" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E262" s="27">
+        <v>54</v>
+      </c>
+      <c r="F262" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G262" s="19"/>
+      <c r="H262" s="19"/>
+      <c r="I262" s="19"/>
+      <c r="J262" s="19"/>
+    </row>
+    <row r="263" spans="4:10" ht="19.2">
+      <c r="D263" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E263" s="27">
+        <v>55</v>
+      </c>
+      <c r="F263" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G263" s="19"/>
+      <c r="H263" s="19"/>
+      <c r="I263" s="19"/>
+      <c r="J263" s="19"/>
+    </row>
+    <row r="264" spans="4:10" ht="19.2">
+      <c r="D264" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E264" s="27">
+        <v>56</v>
+      </c>
+      <c r="F264" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G264" s="19"/>
+      <c r="H264" s="19"/>
+      <c r="I264" s="19"/>
+      <c r="J264" s="19"/>
+    </row>
+    <row r="265" spans="4:10" ht="19.2">
+      <c r="D265" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E265" s="27">
+        <v>57</v>
+      </c>
+      <c r="F265" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G265" s="19"/>
+      <c r="H265" s="19"/>
+      <c r="I265" s="19"/>
+      <c r="J265" s="19"/>
+    </row>
+    <row r="266" spans="4:10" ht="19.2">
+      <c r="D266" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E266" s="27">
+        <v>58</v>
+      </c>
+      <c r="F266" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G266" s="19"/>
+      <c r="H266" s="19"/>
+      <c r="I266" s="19"/>
+      <c r="J266" s="19"/>
+    </row>
+    <row r="267" spans="4:10" ht="19.2">
+      <c r="D267" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E267" s="27">
+        <v>59</v>
+      </c>
+      <c r="F267" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G267" s="19"/>
+      <c r="H267" s="19"/>
+      <c r="I267" s="19"/>
+      <c r="J267" s="19"/>
+    </row>
+    <row r="268" spans="4:10" ht="19.2">
+      <c r="D268" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="E268" s="27">
+        <v>60</v>
+      </c>
+      <c r="F268" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G268" s="19"/>
+      <c r="H268" s="19"/>
+      <c r="I268" s="19"/>
+      <c r="J268" s="19"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix NB202 room naming
</commit_message>
<xml_diff>
--- a/Fees Details 2024-25.xlsx
+++ b/Fees Details 2024-25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HIMANSHU\hostel-management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2C3F09-2845-4288-954F-E69EC021E993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE3B4773-EDF5-4158-8FAC-E83F1829AE87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="428">
   <si>
     <t>ROOMS</t>
   </si>
@@ -1466,9 +1466,6 @@
   </si>
   <si>
     <t>NB202</t>
-  </si>
-  <si>
-    <t>NB 202</t>
   </si>
   <si>
     <t>NB203</t>
@@ -7589,7 +7586,7 @@
     </row>
     <row r="275" spans="4:10" ht="19.2">
       <c r="D275" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E275" s="7">
         <v>3</v>
@@ -7611,7 +7608,7 @@
     </row>
     <row r="277" spans="4:10" ht="19.2">
       <c r="D277" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E277" s="7">
         <v>1</v>
@@ -7634,7 +7631,7 @@
     </row>
     <row r="278" spans="4:10" ht="19.2">
       <c r="D278" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E278" s="7">
         <v>2</v>
@@ -7657,7 +7654,7 @@
     </row>
     <row r="279" spans="4:10" ht="19.2">
       <c r="D279" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E279" s="7">
         <v>3</v>
@@ -7680,7 +7677,7 @@
     </row>
     <row r="280" spans="4:10" ht="19.2">
       <c r="D280" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E280" s="7">
         <v>4</v>
@@ -7703,7 +7700,7 @@
     </row>
     <row r="281" spans="4:10" ht="19.2">
       <c r="D281" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E281" s="7">
         <v>1</v>
@@ -7726,7 +7723,7 @@
     </row>
     <row r="282" spans="4:10" ht="19.2">
       <c r="D282" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E282" s="7">
         <v>2</v>
@@ -7749,7 +7746,7 @@
     </row>
     <row r="283" spans="4:10" ht="19.2">
       <c r="D283" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E283" s="7">
         <v>3</v>
@@ -7772,7 +7769,7 @@
     </row>
     <row r="284" spans="4:10" ht="19.2">
       <c r="D284" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E284" s="7">
         <v>4</v>
@@ -7795,7 +7792,7 @@
     </row>
     <row r="285" spans="4:10" ht="19.2">
       <c r="D285" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E285" s="7">
         <v>1</v>
@@ -7818,7 +7815,7 @@
     </row>
     <row r="286" spans="4:10" ht="19.2">
       <c r="D286" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E286" s="7">
         <v>2</v>
@@ -7841,7 +7838,7 @@
     </row>
     <row r="287" spans="4:10" ht="19.2">
       <c r="D287" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E287" s="7">
         <v>3</v>
@@ -7864,7 +7861,7 @@
     </row>
     <row r="288" spans="4:10" ht="19.2">
       <c r="D288" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E288" s="7">
         <v>4</v>
@@ -7887,7 +7884,7 @@
     </row>
     <row r="289" spans="4:10" ht="19.2">
       <c r="D289" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E289" s="7">
         <v>1</v>
@@ -7910,7 +7907,7 @@
     </row>
     <row r="290" spans="4:10" ht="19.2">
       <c r="D290" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E290" s="7">
         <v>2</v>
@@ -7933,7 +7930,7 @@
     </row>
     <row r="291" spans="4:10" ht="19.2">
       <c r="D291" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E291" s="7">
         <v>3</v>
@@ -7944,7 +7941,7 @@
     </row>
     <row r="292" spans="4:10" ht="19.2">
       <c r="D292" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E292" s="7">
         <v>4</v>
@@ -7955,7 +7952,7 @@
     </row>
     <row r="293" spans="4:10" ht="19.2">
       <c r="D293" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E293" s="7">
         <v>1</v>
@@ -7978,7 +7975,7 @@
     </row>
     <row r="294" spans="4:10" ht="19.2">
       <c r="D294" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E294" s="7">
         <v>2</v>
@@ -8001,7 +7998,7 @@
     </row>
     <row r="295" spans="4:10" ht="19.2">
       <c r="D295" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E295" s="7">
         <v>3</v>
@@ -8024,7 +8021,7 @@
     </row>
     <row r="296" spans="4:10" ht="19.2">
       <c r="D296" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E296" s="7">
         <v>4</v>
@@ -8047,7 +8044,7 @@
     </row>
     <row r="297" spans="4:10" ht="19.2">
       <c r="D297" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E297" s="7">
         <v>1</v>
@@ -8070,7 +8067,7 @@
     </row>
     <row r="298" spans="4:10" ht="19.2">
       <c r="D298" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E298" s="7">
         <v>2</v>
@@ -8093,7 +8090,7 @@
     </row>
     <row r="299" spans="4:10" ht="19.2">
       <c r="D299" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E299" s="7">
         <v>3</v>
@@ -8116,7 +8113,7 @@
     </row>
     <row r="300" spans="4:10" ht="19.2">
       <c r="D300" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E300" s="7">
         <v>4</v>
@@ -8127,7 +8124,7 @@
     </row>
     <row r="301" spans="4:10" ht="19.2">
       <c r="D301" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E301" s="7">
         <v>1</v>
@@ -8150,7 +8147,7 @@
     </row>
     <row r="302" spans="4:10" ht="19.2">
       <c r="D302" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E302" s="7">
         <v>2</v>
@@ -8173,7 +8170,7 @@
     </row>
     <row r="303" spans="4:10" ht="19.2">
       <c r="D303" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E303" s="7">
         <v>3</v>
@@ -8196,7 +8193,7 @@
     </row>
     <row r="304" spans="4:10" ht="19.2">
       <c r="D304" s="3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E304" s="7">
         <v>4</v>
@@ -8219,7 +8216,7 @@
     </row>
     <row r="305" spans="4:10" ht="19.2">
       <c r="D305" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E305" s="7">
         <v>1</v>
@@ -8242,7 +8239,7 @@
     </row>
     <row r="306" spans="4:10" ht="19.2">
       <c r="D306" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E306" s="7">
         <v>2</v>
@@ -8265,7 +8262,7 @@
     </row>
     <row r="307" spans="4:10" ht="19.2">
       <c r="D307" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E307" s="7">
         <v>3</v>
@@ -8288,7 +8285,7 @@
     </row>
     <row r="308" spans="4:10" ht="19.2">
       <c r="D308" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E308" s="7">
         <v>4</v>
@@ -8311,7 +8308,7 @@
     </row>
     <row r="309" spans="4:10" ht="19.2">
       <c r="D309" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E309" s="7">
         <v>1</v>
@@ -8334,7 +8331,7 @@
     </row>
     <row r="310" spans="4:10" ht="19.2">
       <c r="D310" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E310" s="7">
         <v>2</v>
@@ -8357,7 +8354,7 @@
     </row>
     <row r="311" spans="4:10" ht="19.2">
       <c r="D311" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E311" s="7">
         <v>3</v>
@@ -8380,7 +8377,7 @@
     </row>
     <row r="312" spans="4:10" ht="19.2">
       <c r="D312" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E312" s="7">
         <v>4</v>
@@ -8391,7 +8388,7 @@
     </row>
     <row r="313" spans="4:10" ht="19.2">
       <c r="D313" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E313" s="7">
         <v>1</v>
@@ -8414,7 +8411,7 @@
     </row>
     <row r="314" spans="4:10" ht="19.2">
       <c r="D314" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E314" s="7">
         <v>2</v>
@@ -8437,7 +8434,7 @@
     </row>
     <row r="315" spans="4:10" ht="19.2">
       <c r="D315" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E315" s="7">
         <v>3</v>
@@ -8460,7 +8457,7 @@
     </row>
     <row r="316" spans="4:10" ht="19.2">
       <c r="D316" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E316" s="7">
         <v>4</v>
@@ -8483,7 +8480,7 @@
     </row>
     <row r="317" spans="4:10" ht="19.2">
       <c r="D317" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E317" s="7">
         <v>1</v>
@@ -8506,7 +8503,7 @@
     </row>
     <row r="318" spans="4:10" ht="19.2">
       <c r="D318" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E318" s="7">
         <v>2</v>
@@ -8529,7 +8526,7 @@
     </row>
     <row r="319" spans="4:10" ht="19.2">
       <c r="D319" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E319" s="7">
         <v>3</v>
@@ -8552,7 +8549,7 @@
     </row>
     <row r="320" spans="4:10" ht="19.2">
       <c r="D320" s="3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E320" s="7">
         <v>4</v>
@@ -8575,7 +8572,7 @@
     </row>
     <row r="321" spans="4:10" ht="19.2">
       <c r="D321" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E321" s="7">
         <v>1</v>
@@ -8598,7 +8595,7 @@
     </row>
     <row r="322" spans="4:10" ht="19.2">
       <c r="D322" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E322" s="7">
         <v>2</v>
@@ -8621,7 +8618,7 @@
     </row>
     <row r="323" spans="4:10" ht="19.2">
       <c r="D323" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E323" s="7">
         <v>3</v>
@@ -8644,7 +8641,7 @@
     </row>
     <row r="324" spans="4:10" ht="19.2">
       <c r="D324" s="3" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E324" s="7">
         <v>4</v>
@@ -8667,7 +8664,7 @@
     </row>
     <row r="325" spans="4:10" ht="19.2">
       <c r="D325" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E325" s="7">
         <v>1</v>
@@ -8690,7 +8687,7 @@
     </row>
     <row r="326" spans="4:10" ht="19.2">
       <c r="D326" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E326" s="7">
         <v>2</v>
@@ -8713,7 +8710,7 @@
     </row>
     <row r="327" spans="4:10" ht="19.2">
       <c r="D327" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E327" s="7">
         <v>3</v>
@@ -8736,7 +8733,7 @@
     </row>
     <row r="328" spans="4:10" ht="19.2">
       <c r="D328" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="E328" s="7">
         <v>4</v>
@@ -8759,7 +8756,7 @@
     </row>
     <row r="329" spans="4:10" ht="19.2">
       <c r="D329" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E329" s="7">
         <v>1</v>
@@ -8782,7 +8779,7 @@
     </row>
     <row r="330" spans="4:10" ht="19.2">
       <c r="D330" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E330" s="7">
         <v>2</v>
@@ -8805,7 +8802,7 @@
     </row>
     <row r="331" spans="4:10" ht="19.2">
       <c r="D331" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E331" s="7">
         <v>3</v>
@@ -8816,7 +8813,7 @@
     </row>
     <row r="332" spans="4:10" ht="19.2">
       <c r="D332" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E332" s="7">
         <v>4</v>
@@ -8827,7 +8824,7 @@
     </row>
     <row r="333" spans="4:10" ht="19.2">
       <c r="D333" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E333" s="7">
         <v>1</v>
@@ -8850,7 +8847,7 @@
     </row>
     <row r="334" spans="4:10" ht="19.2">
       <c r="D334" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E334" s="7">
         <v>2</v>
@@ -8871,7 +8868,7 @@
     </row>
     <row r="335" spans="4:10" ht="19.2">
       <c r="D335" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E335" s="7">
         <v>3</v>
@@ -8894,7 +8891,7 @@
     </row>
     <row r="336" spans="4:10" ht="19.2">
       <c r="D336" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E336" s="7">
         <v>4</v>
@@ -8905,7 +8902,7 @@
     </row>
     <row r="337" spans="4:10" ht="19.2">
       <c r="D337" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E337" s="7">
         <v>1</v>
@@ -8928,7 +8925,7 @@
     </row>
     <row r="338" spans="4:10" ht="19.2">
       <c r="D338" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E338" s="7">
         <v>2</v>
@@ -8951,7 +8948,7 @@
     </row>
     <row r="339" spans="4:10" ht="19.2">
       <c r="D339" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E339" s="7">
         <v>3</v>
@@ -8962,7 +8959,7 @@
     </row>
     <row r="340" spans="4:10" ht="19.2">
       <c r="D340" s="3" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="E340" s="7">
         <v>4</v>
@@ -8973,7 +8970,7 @@
     </row>
     <row r="341" spans="4:10" ht="19.2">
       <c r="D341" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E341" s="7">
         <v>1</v>
@@ -8996,7 +8993,7 @@
     </row>
     <row r="342" spans="4:10" ht="19.2">
       <c r="D342" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E342" s="7">
         <v>2</v>
@@ -9019,7 +9016,7 @@
     </row>
     <row r="343" spans="4:10" ht="19.2">
       <c r="D343" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E343" s="7">
         <v>3</v>
@@ -9042,7 +9039,7 @@
     </row>
     <row r="344" spans="4:10" ht="19.2">
       <c r="D344" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E344" s="7">
         <v>4</v>
@@ -9065,7 +9062,7 @@
     </row>
     <row r="345" spans="4:10" ht="19.2">
       <c r="D345" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E345" s="7">
         <v>1</v>
@@ -9088,7 +9085,7 @@
     </row>
     <row r="346" spans="4:10" ht="19.2">
       <c r="D346" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E346" s="7">
         <v>2</v>
@@ -9111,7 +9108,7 @@
     </row>
     <row r="347" spans="4:10" ht="19.2">
       <c r="D347" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E347" s="7">
         <v>3</v>
@@ -9134,7 +9131,7 @@
     </row>
     <row r="348" spans="4:10" ht="19.2">
       <c r="D348" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="E348" s="7">
         <v>4</v>
@@ -9145,7 +9142,7 @@
     </row>
     <row r="349" spans="4:10" ht="19.2">
       <c r="D349" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E349" s="7">
         <v>1</v>
@@ -9156,7 +9153,7 @@
     </row>
     <row r="350" spans="4:10" ht="19.2">
       <c r="D350" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E350" s="7">
         <v>2</v>
@@ -9167,7 +9164,7 @@
     </row>
     <row r="351" spans="4:10" ht="19.2">
       <c r="D351" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E351" s="7">
         <v>3</v>
@@ -9178,7 +9175,7 @@
     </row>
     <row r="352" spans="4:10" ht="19.2">
       <c r="D352" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E352" s="7">
         <v>4</v>
@@ -9189,7 +9186,7 @@
     </row>
     <row r="353" spans="4:10" ht="19.2">
       <c r="D353" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E353" s="7">
         <v>1</v>
@@ -9212,7 +9209,7 @@
     </row>
     <row r="354" spans="4:10" ht="19.2">
       <c r="D354" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E354" s="7">
         <v>2</v>
@@ -9235,7 +9232,7 @@
     </row>
     <row r="355" spans="4:10" ht="19.2">
       <c r="D355" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E355" s="7">
         <v>3</v>
@@ -9258,7 +9255,7 @@
     </row>
     <row r="356" spans="4:10" ht="19.2">
       <c r="D356" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E356" s="7">
         <v>4</v>
@@ -9281,7 +9278,7 @@
     </row>
     <row r="357" spans="4:10" ht="19.2">
       <c r="D357" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E357" s="7">
         <v>1</v>
@@ -9304,7 +9301,7 @@
     </row>
     <row r="358" spans="4:10" ht="19.2">
       <c r="D358" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E358" s="7">
         <v>2</v>
@@ -9327,7 +9324,7 @@
     </row>
     <row r="359" spans="4:10" ht="19.2">
       <c r="D359" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E359" s="7">
         <v>3</v>
@@ -9350,7 +9347,7 @@
     </row>
     <row r="360" spans="4:10" ht="19.2">
       <c r="D360" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E360" s="7">
         <v>4</v>
@@ -9361,7 +9358,7 @@
     </row>
     <row r="361" spans="4:10" ht="19.2">
       <c r="D361" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E361" s="7">
         <v>1</v>
@@ -9384,7 +9381,7 @@
     </row>
     <row r="362" spans="4:10" ht="19.2">
       <c r="D362" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E362" s="7">
         <v>2</v>
@@ -9407,7 +9404,7 @@
     </row>
     <row r="363" spans="4:10" ht="19.2">
       <c r="D363" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E363" s="7">
         <v>3</v>
@@ -9430,7 +9427,7 @@
     </row>
     <row r="364" spans="4:10" ht="19.2">
       <c r="D364" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E364" s="7">
         <v>4</v>
@@ -9451,7 +9448,7 @@
     </row>
     <row r="365" spans="4:10" ht="19.2">
       <c r="D365" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E365" s="7">
         <v>1</v>
@@ -9474,7 +9471,7 @@
     </row>
     <row r="366" spans="4:10" ht="19.2">
       <c r="D366" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E366" s="7">
         <v>2</v>
@@ -9497,7 +9494,7 @@
     </row>
     <row r="367" spans="4:10" ht="19.2">
       <c r="D367" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E367" s="7">
         <v>3</v>
@@ -9520,7 +9517,7 @@
     </row>
     <row r="368" spans="4:10" ht="19.2">
       <c r="D368" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E368" s="7">
         <v>4</v>
@@ -9543,7 +9540,7 @@
     </row>
     <row r="369" spans="4:10" ht="19.2">
       <c r="D369" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E369" s="7">
         <v>1</v>
@@ -9566,7 +9563,7 @@
     </row>
     <row r="370" spans="4:10" ht="19.2">
       <c r="D370" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E370" s="7">
         <v>2</v>
@@ -9589,7 +9586,7 @@
     </row>
     <row r="371" spans="4:10" ht="19.2">
       <c r="D371" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E371" s="7">
         <v>3</v>
@@ -9612,7 +9609,7 @@
     </row>
     <row r="372" spans="4:10" ht="19.2">
       <c r="D372" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E372" s="7">
         <v>4</v>
@@ -9633,7 +9630,7 @@
     </row>
     <row r="373" spans="4:10" ht="19.2">
       <c r="D373" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E373" s="7">
         <v>1</v>
@@ -9656,7 +9653,7 @@
     </row>
     <row r="374" spans="4:10" ht="19.2">
       <c r="D374" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E374" s="7">
         <v>2</v>
@@ -9679,7 +9676,7 @@
     </row>
     <row r="375" spans="4:10" ht="19.2">
       <c r="D375" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E375" s="7">
         <v>3</v>
@@ -9702,7 +9699,7 @@
     </row>
     <row r="376" spans="4:10" ht="19.2">
       <c r="D376" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E376" s="7">
         <v>4</v>
@@ -9725,7 +9722,7 @@
     </row>
     <row r="377" spans="4:10" ht="19.2">
       <c r="D377" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E377" s="7">
         <v>1</v>
@@ -9748,7 +9745,7 @@
     </row>
     <row r="378" spans="4:10" ht="19.2">
       <c r="D378" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E378" s="7">
         <v>2</v>
@@ -9771,7 +9768,7 @@
     </row>
     <row r="379" spans="4:10" ht="19.2">
       <c r="D379" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E379" s="7">
         <v>3</v>
@@ -9794,7 +9791,7 @@
     </row>
     <row r="380" spans="4:10" ht="19.2">
       <c r="D380" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E380" s="7">
         <v>4</v>
@@ -9817,7 +9814,7 @@
     </row>
     <row r="381" spans="4:10" ht="19.2">
       <c r="D381" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E381" s="7">
         <v>1</v>
@@ -9840,7 +9837,7 @@
     </row>
     <row r="382" spans="4:10" ht="19.2">
       <c r="D382" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E382" s="7">
         <v>2</v>
@@ -9851,7 +9848,7 @@
     </row>
     <row r="383" spans="4:10" ht="19.2">
       <c r="D383" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E383" s="7">
         <v>3</v>
@@ -9862,7 +9859,7 @@
     </row>
     <row r="384" spans="4:10" ht="19.2">
       <c r="D384" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E384" s="7">
         <v>4</v>
@@ -9873,7 +9870,7 @@
     </row>
     <row r="385" spans="4:10" ht="19.2">
       <c r="D385" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E385" s="7">
         <v>1</v>
@@ -9893,7 +9890,7 @@
     </row>
     <row r="386" spans="4:10" ht="19.2">
       <c r="D386" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E386" s="7">
         <v>2</v>
@@ -9913,7 +9910,7 @@
     </row>
     <row r="387" spans="4:10" ht="19.2">
       <c r="D387" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E387" s="7">
         <v>3</v>
@@ -9933,7 +9930,7 @@
     </row>
     <row r="388" spans="4:10" ht="19.2">
       <c r="D388" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E388" s="7">
         <v>4</v>

</xml_diff>